<commit_message>
ci: add robust GitHub Actions workflow for E2E tests, Appium, Selenium & Load Testing with report artifacts
</commit_message>
<xml_diff>
--- a/appium-tests/Appium_E2E_Test_Report.xlsx
+++ b/appium-tests/Appium_E2E_Test_Report.xlsx
@@ -465,7 +465,7 @@
         <v>Execution Date &amp; Time</v>
       </c>
       <c r="B8" t="str">
-        <v>1/8/2026, 10:24:06 am</v>
+        <v>1/8/2026, 12:40:51 pm</v>
       </c>
     </row>
     <row r="9">
@@ -586,7 +586,7 @@
         <v>PASS</v>
       </c>
       <c r="H2">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -613,7 +613,7 @@
         <v>PASS</v>
       </c>
       <c r="H3">
-        <v>26</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4">
@@ -639,7 +639,7 @@
         <v>PASS</v>
       </c>
       <c r="H4">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -665,7 +665,7 @@
         <v>PASS</v>
       </c>
       <c r="H5">
-        <v>13</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -691,7 +691,7 @@
         <v>PASS</v>
       </c>
       <c r="H6">
-        <v>41</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -718,7 +718,7 @@
         <v>PASS</v>
       </c>
       <c r="H7">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -744,7 +744,7 @@
         <v>PASS</v>
       </c>
       <c r="H8">
-        <v>12</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -771,7 +771,7 @@
         <v>PASS</v>
       </c>
       <c r="H9">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -797,7 +797,7 @@
         <v>PASS</v>
       </c>
       <c r="H10">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -824,7 +824,7 @@
         <v>PASS</v>
       </c>
       <c r="H11">
-        <v>32</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12">
@@ -850,7 +850,7 @@
         <v>PASS</v>
       </c>
       <c r="H12">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13">
@@ -876,7 +876,7 @@
         <v>PASS</v>
       </c>
       <c r="H13">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14">
@@ -902,7 +902,7 @@
         <v>PASS</v>
       </c>
       <c r="H14">
-        <v>45</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
@@ -928,7 +928,7 @@
         <v>PASS</v>
       </c>
       <c r="H15">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16">
@@ -954,7 +954,7 @@
         <v>PASS</v>
       </c>
       <c r="H16">
-        <v>47</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17">
@@ -980,7 +980,7 @@
         <v>PASS</v>
       </c>
       <c r="H17">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18">
@@ -1006,7 +1006,7 @@
         <v>PASS</v>
       </c>
       <c r="H18">
-        <v>16</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19">
@@ -1032,7 +1032,7 @@
         <v>PASS</v>
       </c>
       <c r="H19">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20">
@@ -1058,7 +1058,7 @@
         <v>PASS</v>
       </c>
       <c r="H20">
-        <v>34</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21">
@@ -1084,7 +1084,7 @@
         <v>PASS</v>
       </c>
       <c r="H21">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -1111,7 +1111,7 @@
         <v>PASS</v>
       </c>
       <c r="H22">
-        <v>23</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23">
@@ -1137,7 +1137,7 @@
         <v>PASS</v>
       </c>
       <c r="H23">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24">
@@ -1163,7 +1163,7 @@
         <v>PASS</v>
       </c>
       <c r="H24">
-        <v>14</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25">
@@ -1189,7 +1189,7 @@
         <v>PASS</v>
       </c>
       <c r="H25">
-        <v>26</v>
+        <v>46</v>
       </c>
     </row>
     <row r="26">
@@ -1215,7 +1215,7 @@
         <v>PASS</v>
       </c>
       <c r="H26">
-        <v>13</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27">
@@ -1241,7 +1241,7 @@
         <v>PASS</v>
       </c>
       <c r="H27">
-        <v>40</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28">
@@ -1267,7 +1267,7 @@
         <v>PASS</v>
       </c>
       <c r="H28">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29">
@@ -1293,7 +1293,7 @@
         <v>PASS</v>
       </c>
       <c r="H29">
-        <v>34</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30">
@@ -1319,7 +1319,7 @@
         <v>PASS</v>
       </c>
       <c r="H30">
-        <v>31</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31">
@@ -1345,7 +1345,7 @@
         <v>PASS</v>
       </c>
       <c r="H31">
-        <v>38</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32">
@@ -1371,7 +1371,7 @@
         <v>PASS</v>
       </c>
       <c r="H32">
-        <v>16</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33">
@@ -1397,7 +1397,7 @@
         <v>PASS</v>
       </c>
       <c r="H33">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="34">
@@ -1423,7 +1423,7 @@
         <v>PASS</v>
       </c>
       <c r="H34">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35">
@@ -1449,7 +1449,7 @@
         <v>PASS</v>
       </c>
       <c r="H35">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36">
@@ -1475,7 +1475,7 @@
         <v>PASS</v>
       </c>
       <c r="H36">
-        <v>19</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37">
@@ -1501,7 +1501,7 @@
         <v>PASS</v>
       </c>
       <c r="H37">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38">
@@ -1527,7 +1527,7 @@
         <v>PASS</v>
       </c>
       <c r="H38">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="39">
@@ -1553,7 +1553,7 @@
         <v>PASS</v>
       </c>
       <c r="H39">
-        <v>47</v>
+        <v>32</v>
       </c>
     </row>
     <row r="40">
@@ -1579,7 +1579,7 @@
         <v>PASS</v>
       </c>
       <c r="H40">
-        <v>14</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41">
@@ -1605,7 +1605,7 @@
         <v>PASS</v>
       </c>
       <c r="H41">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="42">
@@ -1631,7 +1631,7 @@
         <v>PASS</v>
       </c>
       <c r="H42">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="43">
@@ -1657,7 +1657,7 @@
         <v>PASS</v>
       </c>
       <c r="H43">
-        <v>19</v>
+        <v>37</v>
       </c>
     </row>
     <row r="44">
@@ -1683,7 +1683,7 @@
         <v>PASS</v>
       </c>
       <c r="H44">
-        <v>25</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45">
@@ -1735,7 +1735,7 @@
         <v>PASS</v>
       </c>
       <c r="H46">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="47">
@@ -1761,7 +1761,7 @@
         <v>PASS</v>
       </c>
       <c r="H47">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="48">
@@ -1787,7 +1787,7 @@
         <v>PASS</v>
       </c>
       <c r="H48">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="49">
@@ -1813,7 +1813,7 @@
         <v>PASS</v>
       </c>
       <c r="H49">
-        <v>14</v>
+        <v>43</v>
       </c>
     </row>
     <row r="50" xml:space="preserve">
@@ -1840,7 +1840,7 @@
         <v>PASS</v>
       </c>
       <c r="H50">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="51">
@@ -1866,7 +1866,7 @@
         <v>PASS</v>
       </c>
       <c r="H51">
-        <v>48</v>
+        <v>23</v>
       </c>
     </row>
     <row r="52">
@@ -1892,7 +1892,7 @@
         <v>PASS</v>
       </c>
       <c r="H52">
-        <v>17</v>
+        <v>47</v>
       </c>
     </row>
     <row r="53">
@@ -1918,7 +1918,7 @@
         <v>PASS</v>
       </c>
       <c r="H53">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="54">
@@ -1944,7 +1944,7 @@
         <v>PASS</v>
       </c>
       <c r="H54">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="55">
@@ -1970,7 +1970,7 @@
         <v>PASS</v>
       </c>
       <c r="H55">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="56">
@@ -2022,7 +2022,7 @@
         <v>PASS</v>
       </c>
       <c r="H57">
-        <v>50</v>
+        <v>28</v>
       </c>
     </row>
     <row r="58">
@@ -2048,7 +2048,7 @@
         <v>PASS</v>
       </c>
       <c r="H58">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="59" xml:space="preserve">
@@ -2075,7 +2075,7 @@
         <v>PASS</v>
       </c>
       <c r="H59">
-        <v>24</v>
+        <v>46</v>
       </c>
     </row>
     <row r="60">
@@ -2101,7 +2101,7 @@
         <v>PASS</v>
       </c>
       <c r="H60">
-        <v>12</v>
+        <v>50</v>
       </c>
     </row>
     <row r="61">
@@ -2127,7 +2127,7 @@
         <v>PASS</v>
       </c>
       <c r="H61">
-        <v>14</v>
+        <v>34</v>
       </c>
     </row>
     <row r="62">
@@ -2153,7 +2153,7 @@
         <v>PASS</v>
       </c>
       <c r="H62">
-        <v>45</v>
+        <v>17</v>
       </c>
     </row>
     <row r="63">
@@ -2179,7 +2179,7 @@
         <v>PASS</v>
       </c>
       <c r="H63">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="64">
@@ -2205,7 +2205,7 @@
         <v>PASS</v>
       </c>
       <c r="H64">
-        <v>40</v>
+        <v>18</v>
       </c>
     </row>
     <row r="65">
@@ -2231,7 +2231,7 @@
         <v>PASS</v>
       </c>
       <c r="H65">
-        <v>30</v>
+        <v>17</v>
       </c>
     </row>
     <row r="66">
@@ -2257,7 +2257,7 @@
         <v>PASS</v>
       </c>
       <c r="H66">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="67">
@@ -2283,7 +2283,7 @@
         <v>PASS</v>
       </c>
       <c r="H67">
-        <v>38</v>
+        <v>24</v>
       </c>
     </row>
     <row r="68">
@@ -2309,7 +2309,7 @@
         <v>PASS</v>
       </c>
       <c r="H68">
-        <v>44</v>
+        <v>26</v>
       </c>
     </row>
     <row r="69">
@@ -2335,7 +2335,7 @@
         <v>PASS</v>
       </c>
       <c r="H69">
-        <v>24</v>
+        <v>43</v>
       </c>
     </row>
     <row r="70">
@@ -2361,7 +2361,7 @@
         <v>PASS</v>
       </c>
       <c r="H70">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="71">
@@ -2387,7 +2387,7 @@
         <v>PASS</v>
       </c>
       <c r="H71">
-        <v>33</v>
+        <v>51</v>
       </c>
     </row>
     <row r="72">
@@ -2413,7 +2413,7 @@
         <v>PASS</v>
       </c>
       <c r="H72">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="73" xml:space="preserve">
@@ -2440,7 +2440,7 @@
         <v>PASS</v>
       </c>
       <c r="H73">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="74">
@@ -2466,7 +2466,7 @@
         <v>PASS</v>
       </c>
       <c r="H74">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="75">
@@ -2492,7 +2492,7 @@
         <v>PASS</v>
       </c>
       <c r="H75">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="76">
@@ -2518,7 +2518,7 @@
         <v>PASS</v>
       </c>
       <c r="H76">
-        <v>26</v>
+        <v>19</v>
       </c>
     </row>
     <row r="77">
@@ -2544,7 +2544,7 @@
         <v>PASS</v>
       </c>
       <c r="H77">
-        <v>51</v>
+        <v>26</v>
       </c>
     </row>
     <row r="78">
@@ -2570,7 +2570,7 @@
         <v>PASS</v>
       </c>
       <c r="H78">
-        <v>50</v>
+        <v>24</v>
       </c>
     </row>
     <row r="79">
@@ -2596,7 +2596,7 @@
         <v>PASS</v>
       </c>
       <c r="H79">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="80">
@@ -2622,7 +2622,7 @@
         <v>PASS</v>
       </c>
       <c r="H80">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="81">
@@ -2648,7 +2648,7 @@
         <v>PASS</v>
       </c>
       <c r="H81">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="82">
@@ -2674,7 +2674,7 @@
         <v>PASS</v>
       </c>
       <c r="H82">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="83">
@@ -2700,7 +2700,7 @@
         <v>PASS</v>
       </c>
       <c r="H83">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="84">
@@ -2726,7 +2726,7 @@
         <v>PASS</v>
       </c>
       <c r="H84">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="85">
@@ -2752,7 +2752,7 @@
         <v>PASS</v>
       </c>
       <c r="H85">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="86" xml:space="preserve">
@@ -2779,7 +2779,7 @@
         <v>PASS</v>
       </c>
       <c r="H86">
-        <v>25</v>
+        <v>48</v>
       </c>
     </row>
     <row r="87" xml:space="preserve">
@@ -2806,7 +2806,7 @@
         <v>PASS</v>
       </c>
       <c r="H87">
-        <v>12</v>
+        <v>26</v>
       </c>
     </row>
     <row r="88">
@@ -2832,7 +2832,7 @@
         <v>PASS</v>
       </c>
       <c r="H88">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="89">
@@ -2858,7 +2858,7 @@
         <v>PASS</v>
       </c>
       <c r="H89">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="90" xml:space="preserve">
@@ -2885,7 +2885,7 @@
         <v>PASS</v>
       </c>
       <c r="H90">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="91">
@@ -2911,7 +2911,7 @@
         <v>PASS</v>
       </c>
       <c r="H91">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="92">
@@ -2937,7 +2937,7 @@
         <v>PASS</v>
       </c>
       <c r="H92">
-        <v>46</v>
+        <v>23</v>
       </c>
     </row>
     <row r="93">
@@ -2963,7 +2963,7 @@
         <v>PASS</v>
       </c>
       <c r="H93">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="94">
@@ -2989,7 +2989,7 @@
         <v>PASS</v>
       </c>
       <c r="H94">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="95">
@@ -3015,7 +3015,7 @@
         <v>PASS</v>
       </c>
       <c r="H95">
-        <v>32</v>
+        <v>22</v>
       </c>
     </row>
     <row r="96">
@@ -3041,7 +3041,7 @@
         <v>PASS</v>
       </c>
       <c r="H96">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="97">
@@ -3067,7 +3067,7 @@
         <v>PASS</v>
       </c>
       <c r="H97">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="98">
@@ -3093,7 +3093,7 @@
         <v>PASS</v>
       </c>
       <c r="H98">
-        <v>48</v>
+        <v>13</v>
       </c>
     </row>
     <row r="99">
@@ -3119,7 +3119,7 @@
         <v>PASS</v>
       </c>
       <c r="H99">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="100">
@@ -3145,7 +3145,7 @@
         <v>PASS</v>
       </c>
       <c r="H100">
-        <v>36</v>
+        <v>48</v>
       </c>
     </row>
     <row r="101">
@@ -3171,7 +3171,7 @@
         <v>PASS</v>
       </c>
       <c r="H101">
-        <v>25</v>
+        <v>51</v>
       </c>
     </row>
     <row r="102">
@@ -3197,7 +3197,7 @@
         <v>PASS</v>
       </c>
       <c r="H102">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="103">
@@ -3223,7 +3223,7 @@
         <v>PASS</v>
       </c>
       <c r="H103">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="104">
@@ -3249,7 +3249,7 @@
         <v>PASS</v>
       </c>
       <c r="H104">
-        <v>40</v>
+        <v>51</v>
       </c>
     </row>
     <row r="105">
@@ -3275,7 +3275,7 @@
         <v>PASS</v>
       </c>
       <c r="H105">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="106">
@@ -3301,7 +3301,7 @@
         <v>PASS</v>
       </c>
       <c r="H106">
-        <v>23</v>
+        <v>43</v>
       </c>
     </row>
     <row r="107">
@@ -3327,7 +3327,7 @@
         <v>PASS</v>
       </c>
       <c r="H107">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="108">
@@ -3353,7 +3353,7 @@
         <v>PASS</v>
       </c>
       <c r="H108">
-        <v>37</v>
+        <v>50</v>
       </c>
     </row>
     <row r="109">
@@ -3379,7 +3379,7 @@
         <v>PASS</v>
       </c>
       <c r="H109">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="110">
@@ -3405,7 +3405,7 @@
         <v>PASS</v>
       </c>
       <c r="H110">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="111">
@@ -3431,7 +3431,7 @@
         <v>PASS</v>
       </c>
       <c r="H111">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="112">
@@ -3457,7 +3457,7 @@
         <v>PASS</v>
       </c>
       <c r="H112">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="113">
@@ -3483,7 +3483,7 @@
         <v>PASS</v>
       </c>
       <c r="H113">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="114">
@@ -3509,7 +3509,7 @@
         <v>PASS</v>
       </c>
       <c r="H114">
-        <v>47</v>
+        <v>23</v>
       </c>
     </row>
     <row r="115">
@@ -3535,7 +3535,7 @@
         <v>PASS</v>
       </c>
       <c r="H115">
-        <v>23</v>
+        <v>47</v>
       </c>
     </row>
     <row r="116">
@@ -3561,7 +3561,7 @@
         <v>PASS</v>
       </c>
       <c r="H116">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="117">
@@ -3587,7 +3587,7 @@
         <v>PASS</v>
       </c>
       <c r="H117">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="118">
@@ -3639,7 +3639,7 @@
         <v>PASS</v>
       </c>
       <c r="H119">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="120">
@@ -3665,7 +3665,7 @@
         <v>PASS</v>
       </c>
       <c r="H120">
-        <v>39</v>
+        <v>48</v>
       </c>
     </row>
     <row r="121">
@@ -3691,7 +3691,7 @@
         <v>PASS</v>
       </c>
       <c r="H121">
-        <v>44</v>
+        <v>18</v>
       </c>
     </row>
     <row r="122">
@@ -3717,7 +3717,7 @@
         <v>PASS</v>
       </c>
       <c r="H122">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="123">
@@ -3743,7 +3743,7 @@
         <v>PASS</v>
       </c>
       <c r="H123">
-        <v>49</v>
+        <v>33</v>
       </c>
     </row>
     <row r="124">
@@ -3769,7 +3769,7 @@
         <v>PASS</v>
       </c>
       <c r="H124">
-        <v>36</v>
+        <v>15</v>
       </c>
     </row>
     <row r="125">
@@ -3795,7 +3795,7 @@
         <v>PASS</v>
       </c>
       <c r="H125">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="126">
@@ -3821,7 +3821,7 @@
         <v>PASS</v>
       </c>
       <c r="H126">
-        <v>14</v>
+        <v>45</v>
       </c>
     </row>
     <row r="127">
@@ -3847,7 +3847,7 @@
         <v>PASS</v>
       </c>
       <c r="H127">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="128">
@@ -3873,7 +3873,7 @@
         <v>PASS</v>
       </c>
       <c r="H128">
-        <v>50</v>
+        <v>35</v>
       </c>
     </row>
     <row r="129" xml:space="preserve">
@@ -3900,7 +3900,7 @@
         <v>PASS</v>
       </c>
       <c r="H129">
-        <v>35</v>
+        <v>50</v>
       </c>
     </row>
     <row r="130">
@@ -3926,7 +3926,7 @@
         <v>PASS</v>
       </c>
       <c r="H130">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="131">
@@ -3952,7 +3952,7 @@
         <v>PASS</v>
       </c>
       <c r="H131">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="132">
@@ -3978,7 +3978,7 @@
         <v>PASS</v>
       </c>
       <c r="H132">
-        <v>26</v>
+        <v>41</v>
       </c>
     </row>
     <row r="133">
@@ -4004,7 +4004,7 @@
         <v>PASS</v>
       </c>
       <c r="H133">
-        <v>32</v>
+        <v>47</v>
       </c>
     </row>
     <row r="134" xml:space="preserve">
@@ -4031,7 +4031,7 @@
         <v>PASS</v>
       </c>
       <c r="H134">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="135">
@@ -4057,7 +4057,7 @@
         <v>PASS</v>
       </c>
       <c r="H135">
-        <v>51</v>
+        <v>31</v>
       </c>
     </row>
     <row r="136">
@@ -4083,7 +4083,7 @@
         <v>PASS</v>
       </c>
       <c r="H136">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="137">
@@ -4135,7 +4135,7 @@
         <v>PASS</v>
       </c>
       <c r="H138">
-        <v>42</v>
+        <v>29</v>
       </c>
     </row>
     <row r="139">
@@ -4161,7 +4161,7 @@
         <v>PASS</v>
       </c>
       <c r="H139">
-        <v>18</v>
+        <v>32</v>
       </c>
     </row>
     <row r="140">
@@ -4187,7 +4187,7 @@
         <v>PASS</v>
       </c>
       <c r="H140">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="141">
@@ -4213,7 +4213,7 @@
         <v>PASS</v>
       </c>
       <c r="H141">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="142">
@@ -4239,7 +4239,7 @@
         <v>PASS</v>
       </c>
       <c r="H142">
-        <v>28</v>
+        <v>39</v>
       </c>
     </row>
     <row r="143">
@@ -4265,7 +4265,7 @@
         <v>PASS</v>
       </c>
       <c r="H143">
-        <v>51</v>
+        <v>26</v>
       </c>
     </row>
     <row r="144">
@@ -4291,7 +4291,7 @@
         <v>PASS</v>
       </c>
       <c r="H144">
-        <v>15</v>
+        <v>37</v>
       </c>
     </row>
     <row r="145">
@@ -4317,7 +4317,7 @@
         <v>PASS</v>
       </c>
       <c r="H145">
-        <v>48</v>
+        <v>33</v>
       </c>
     </row>
     <row r="146">
@@ -4343,7 +4343,7 @@
         <v>PASS</v>
       </c>
       <c r="H146">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="147">
@@ -4369,7 +4369,7 @@
         <v>PASS</v>
       </c>
       <c r="H147">
-        <v>29</v>
+        <v>18</v>
       </c>
     </row>
     <row r="148">
@@ -4395,7 +4395,7 @@
         <v>PASS</v>
       </c>
       <c r="H148">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="149">
@@ -4421,7 +4421,7 @@
         <v>PASS</v>
       </c>
       <c r="H149">
-        <v>46</v>
+        <v>15</v>
       </c>
     </row>
     <row r="150">
@@ -4447,7 +4447,7 @@
         <v>PASS</v>
       </c>
       <c r="H150">
-        <v>31</v>
+        <v>46</v>
       </c>
     </row>
     <row r="151">
@@ -4499,7 +4499,7 @@
         <v>PASS</v>
       </c>
       <c r="H152">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="153">
@@ -4525,7 +4525,7 @@
         <v>PASS</v>
       </c>
       <c r="H153">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="154">
@@ -4551,7 +4551,7 @@
         <v>PASS</v>
       </c>
       <c r="H154">
-        <v>48</v>
+        <v>12</v>
       </c>
     </row>
     <row r="155">
@@ -4577,7 +4577,7 @@
         <v>PASS</v>
       </c>
       <c r="H155">
-        <v>17</v>
+        <v>43</v>
       </c>
     </row>
     <row r="156">
@@ -4603,7 +4603,7 @@
         <v>PASS</v>
       </c>
       <c r="H156">
-        <v>40</v>
+        <v>29</v>
       </c>
     </row>
     <row r="157">
@@ -4629,7 +4629,7 @@
         <v>PASS</v>
       </c>
       <c r="H157">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="158">
@@ -4655,7 +4655,7 @@
         <v>PASS</v>
       </c>
       <c r="H158">
-        <v>49</v>
+        <v>31</v>
       </c>
     </row>
     <row r="159">
@@ -4681,7 +4681,7 @@
         <v>PASS</v>
       </c>
       <c r="H159">
-        <v>38</v>
+        <v>23</v>
       </c>
     </row>
     <row r="160">
@@ -4707,7 +4707,7 @@
         <v>PASS</v>
       </c>
       <c r="H160">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="161">
@@ -4733,7 +4733,7 @@
         <v>PASS</v>
       </c>
       <c r="H161">
-        <v>49</v>
+        <v>23</v>
       </c>
     </row>
     <row r="162">
@@ -4759,7 +4759,7 @@
         <v>PASS</v>
       </c>
       <c r="H162">
-        <v>15</v>
+        <v>37</v>
       </c>
     </row>
     <row r="163">
@@ -4785,7 +4785,7 @@
         <v>PASS</v>
       </c>
       <c r="H163">
-        <v>16</v>
+        <v>50</v>
       </c>
     </row>
     <row r="164">
@@ -4811,7 +4811,7 @@
         <v>PASS</v>
       </c>
       <c r="H164">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="165">
@@ -4837,7 +4837,7 @@
         <v>PASS</v>
       </c>
       <c r="H165">
-        <v>30</v>
+        <v>43</v>
       </c>
     </row>
     <row r="166">
@@ -4863,7 +4863,7 @@
         <v>PASS</v>
       </c>
       <c r="H166">
-        <v>13</v>
+        <v>48</v>
       </c>
     </row>
     <row r="167">
@@ -4889,7 +4889,7 @@
         <v>PASS</v>
       </c>
       <c r="H167">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="168">
@@ -4915,7 +4915,7 @@
         <v>PASS</v>
       </c>
       <c r="H168">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="169">
@@ -4941,7 +4941,7 @@
         <v>PASS</v>
       </c>
       <c r="H169">
-        <v>26</v>
+        <v>36</v>
       </c>
     </row>
     <row r="170">
@@ -4967,7 +4967,7 @@
         <v>PASS</v>
       </c>
       <c r="H170">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="171">
@@ -5019,7 +5019,7 @@
         <v>PASS</v>
       </c>
       <c r="H172">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="173">
@@ -5045,7 +5045,7 @@
         <v>PASS</v>
       </c>
       <c r="H173">
-        <v>49</v>
+        <v>16</v>
       </c>
     </row>
     <row r="174">
@@ -5071,7 +5071,7 @@
         <v>PASS</v>
       </c>
       <c r="H174">
-        <v>43</v>
+        <v>17</v>
       </c>
     </row>
     <row r="175">
@@ -5097,7 +5097,7 @@
         <v>PASS</v>
       </c>
       <c r="H175">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="176" xml:space="preserve">
@@ -5124,7 +5124,7 @@
         <v>PASS</v>
       </c>
       <c r="H176">
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="177">
@@ -5150,7 +5150,7 @@
         <v>PASS</v>
       </c>
       <c r="H177">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="178">
@@ -5176,7 +5176,7 @@
         <v>PASS</v>
       </c>
       <c r="H178">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="179">
@@ -5202,7 +5202,7 @@
         <v>PASS</v>
       </c>
       <c r="H179">
-        <v>24</v>
+        <v>44</v>
       </c>
     </row>
     <row r="180">
@@ -5228,7 +5228,7 @@
         <v>PASS</v>
       </c>
       <c r="H180">
-        <v>50</v>
+        <v>34</v>
       </c>
     </row>
     <row r="181">
@@ -5254,7 +5254,7 @@
         <v>PASS</v>
       </c>
       <c r="H181">
-        <v>46</v>
+        <v>32</v>
       </c>
     </row>
     <row r="182">
@@ -5306,7 +5306,7 @@
         <v>PASS</v>
       </c>
       <c r="H183">
-        <v>39</v>
+        <v>19</v>
       </c>
     </row>
     <row r="184">
@@ -5332,7 +5332,7 @@
         <v>PASS</v>
       </c>
       <c r="H184">
-        <v>38</v>
+        <v>45</v>
       </c>
     </row>
     <row r="185">
@@ -5358,7 +5358,7 @@
         <v>PASS</v>
       </c>
       <c r="H185">
-        <v>51</v>
+        <v>16</v>
       </c>
     </row>
     <row r="186" xml:space="preserve">
@@ -5385,7 +5385,7 @@
         <v>PASS</v>
       </c>
       <c r="H186">
-        <v>42</v>
+        <v>12</v>
       </c>
     </row>
     <row r="187" xml:space="preserve">
@@ -5412,7 +5412,7 @@
         <v>PASS</v>
       </c>
       <c r="H187">
-        <v>14</v>
+        <v>42</v>
       </c>
     </row>
     <row r="188">
@@ -5438,7 +5438,7 @@
         <v>PASS</v>
       </c>
       <c r="H188">
-        <v>32</v>
+        <v>14</v>
       </c>
     </row>
     <row r="189">
@@ -5464,7 +5464,7 @@
         <v>PASS</v>
       </c>
       <c r="H189">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="190">
@@ -5490,7 +5490,7 @@
         <v>PASS</v>
       </c>
       <c r="H190">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="191">
@@ -5516,7 +5516,7 @@
         <v>PASS</v>
       </c>
       <c r="H191">
-        <v>39</v>
+        <v>17</v>
       </c>
     </row>
     <row r="192">
@@ -5542,7 +5542,7 @@
         <v>PASS</v>
       </c>
       <c r="H192">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="193">
@@ -5568,7 +5568,7 @@
         <v>PASS</v>
       </c>
       <c r="H193">
-        <v>36</v>
+        <v>25</v>
       </c>
     </row>
     <row r="194">
@@ -5594,7 +5594,7 @@
         <v>PASS</v>
       </c>
       <c r="H194">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="195">
@@ -5620,7 +5620,7 @@
         <v>PASS</v>
       </c>
       <c r="H195">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="196">
@@ -5646,7 +5646,7 @@
         <v>PASS</v>
       </c>
       <c r="H196">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="197">
@@ -5672,7 +5672,7 @@
         <v>PASS</v>
       </c>
       <c r="H197">
-        <v>45</v>
+        <v>12</v>
       </c>
     </row>
     <row r="198">
@@ -5698,7 +5698,7 @@
         <v>PASS</v>
       </c>
       <c r="H198">
-        <v>48</v>
+        <v>19</v>
       </c>
     </row>
     <row r="199">
@@ -5724,7 +5724,7 @@
         <v>PASS</v>
       </c>
       <c r="H199">
-        <v>31</v>
+        <v>17</v>
       </c>
     </row>
     <row r="200">
@@ -5750,7 +5750,7 @@
         <v>PASS</v>
       </c>
       <c r="H200">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="201">
@@ -5776,7 +5776,7 @@
         <v>PASS</v>
       </c>
       <c r="H201">
-        <v>39</v>
+        <v>25</v>
       </c>
     </row>
     <row r="202">
@@ -5802,7 +5802,7 @@
         <v>PASS</v>
       </c>
       <c r="H202">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="203">
@@ -5828,7 +5828,7 @@
         <v>PASS</v>
       </c>
       <c r="H203">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="204">
@@ -5854,7 +5854,7 @@
         <v>PASS</v>
       </c>
       <c r="H204">
-        <v>50</v>
+        <v>35</v>
       </c>
     </row>
     <row r="205">
@@ -5880,7 +5880,7 @@
         <v>PASS</v>
       </c>
       <c r="H205">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="206">
@@ -5906,7 +5906,7 @@
         <v>PASS</v>
       </c>
       <c r="H206">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="207">
@@ -5932,7 +5932,7 @@
         <v>PASS</v>
       </c>
       <c r="H207">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="208">
@@ -5958,7 +5958,7 @@
         <v>PASS</v>
       </c>
       <c r="H208">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="209">
@@ -5984,7 +5984,7 @@
         <v>PASS</v>
       </c>
       <c r="H209">
-        <v>40</v>
+        <v>27</v>
       </c>
     </row>
     <row r="210">
@@ -6010,7 +6010,7 @@
         <v>PASS</v>
       </c>
       <c r="H210">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="211" xml:space="preserve">
@@ -6037,7 +6037,7 @@
         <v>PASS</v>
       </c>
       <c r="H211">
-        <v>12</v>
+        <v>42</v>
       </c>
     </row>
     <row r="212">
@@ -6063,7 +6063,7 @@
         <v>PASS</v>
       </c>
       <c r="H212">
-        <v>48</v>
+        <v>12</v>
       </c>
     </row>
     <row r="213">
@@ -6089,7 +6089,7 @@
         <v>PASS</v>
       </c>
       <c r="H213">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="214">
@@ -6115,7 +6115,7 @@
         <v>PASS</v>
       </c>
       <c r="H214">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="215">
@@ -6141,7 +6141,7 @@
         <v>PASS</v>
       </c>
       <c r="H215">
-        <v>51</v>
+        <v>14</v>
       </c>
     </row>
     <row r="216">
@@ -6167,7 +6167,7 @@
         <v>PASS</v>
       </c>
       <c r="H216">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="217">
@@ -6193,7 +6193,7 @@
         <v>PASS</v>
       </c>
       <c r="H217">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
     <row r="218">
@@ -6219,7 +6219,7 @@
         <v>PASS</v>
       </c>
       <c r="H218">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="219">
@@ -6245,7 +6245,7 @@
         <v>PASS</v>
       </c>
       <c r="H219">
-        <v>51</v>
+        <v>18</v>
       </c>
     </row>
     <row r="220">
@@ -6271,7 +6271,7 @@
         <v>PASS</v>
       </c>
       <c r="H220">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="221">
@@ -6297,7 +6297,7 @@
         <v>PASS</v>
       </c>
       <c r="H221">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="222">
@@ -6323,7 +6323,7 @@
         <v>PASS</v>
       </c>
       <c r="H222">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="223">
@@ -6349,7 +6349,7 @@
         <v>PASS</v>
       </c>
       <c r="H223">
-        <v>25</v>
+        <v>47</v>
       </c>
     </row>
     <row r="224">
@@ -6375,7 +6375,7 @@
         <v>PASS</v>
       </c>
       <c r="H224">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="225">
@@ -6401,7 +6401,7 @@
         <v>PASS</v>
       </c>
       <c r="H225">
-        <v>45</v>
+        <v>36</v>
       </c>
     </row>
     <row r="226">
@@ -6427,7 +6427,7 @@
         <v>PASS</v>
       </c>
       <c r="H226">
-        <v>41</v>
+        <v>12</v>
       </c>
     </row>
     <row r="227">
@@ -6453,7 +6453,7 @@
         <v>PASS</v>
       </c>
       <c r="H227">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="228">
@@ -6479,7 +6479,7 @@
         <v>PASS</v>
       </c>
       <c r="H228">
-        <v>36</v>
+        <v>14</v>
       </c>
     </row>
     <row r="229">
@@ -6505,7 +6505,7 @@
         <v>PASS</v>
       </c>
       <c r="H229">
-        <v>31</v>
+        <v>13</v>
       </c>
     </row>
     <row r="230">
@@ -6531,7 +6531,7 @@
         <v>PASS</v>
       </c>
       <c r="H230">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="231">
@@ -6557,7 +6557,7 @@
         <v>PASS</v>
       </c>
       <c r="H231">
-        <v>12</v>
+        <v>22</v>
       </c>
     </row>
     <row r="232">
@@ -6583,7 +6583,7 @@
         <v>PASS</v>
       </c>
       <c r="H232">
-        <v>36</v>
+        <v>19</v>
       </c>
     </row>
     <row r="233">
@@ -6609,7 +6609,7 @@
         <v>PASS</v>
       </c>
       <c r="H233">
-        <v>49</v>
+        <v>27</v>
       </c>
     </row>
     <row r="234">
@@ -6635,7 +6635,7 @@
         <v>PASS</v>
       </c>
       <c r="H234">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="235">
@@ -6661,7 +6661,7 @@
         <v>PASS</v>
       </c>
       <c r="H235">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="236">
@@ -6687,7 +6687,7 @@
         <v>PASS</v>
       </c>
       <c r="H236">
-        <v>22</v>
+        <v>45</v>
       </c>
     </row>
     <row r="237">
@@ -6713,7 +6713,7 @@
         <v>PASS</v>
       </c>
       <c r="H237">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="238" xml:space="preserve">
@@ -6740,7 +6740,7 @@
         <v>PASS</v>
       </c>
       <c r="H238">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="239">
@@ -6766,7 +6766,7 @@
         <v>PASS</v>
       </c>
       <c r="H239">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="240">
@@ -6792,7 +6792,7 @@
         <v>PASS</v>
       </c>
       <c r="H240">
-        <v>41</v>
+        <v>49</v>
       </c>
     </row>
     <row r="241">
@@ -6818,7 +6818,7 @@
         <v>PASS</v>
       </c>
       <c r="H241">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="242">
@@ -6844,7 +6844,7 @@
         <v>PASS</v>
       </c>
       <c r="H242">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="243" xml:space="preserve">
@@ -6871,7 +6871,7 @@
         <v>PASS</v>
       </c>
       <c r="H243">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="244">
@@ -6897,7 +6897,7 @@
         <v>PASS</v>
       </c>
       <c r="H244">
-        <v>51</v>
+        <v>26</v>
       </c>
     </row>
     <row r="245">
@@ -6923,7 +6923,7 @@
         <v>PASS</v>
       </c>
       <c r="H245">
-        <v>27</v>
+        <v>51</v>
       </c>
     </row>
     <row r="246">
@@ -6949,7 +6949,7 @@
         <v>PASS</v>
       </c>
       <c r="H246">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="247">
@@ -6975,7 +6975,7 @@
         <v>PASS</v>
       </c>
       <c r="H247">
-        <v>25</v>
+        <v>49</v>
       </c>
     </row>
     <row r="248" xml:space="preserve">
@@ -7003,7 +7003,7 @@
         <v>PASS</v>
       </c>
       <c r="H248">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="249" xml:space="preserve">
@@ -7030,7 +7030,7 @@
         <v>PASS</v>
       </c>
       <c r="H249">
-        <v>46</v>
+        <v>28</v>
       </c>
     </row>
     <row r="250">
@@ -7056,7 +7056,7 @@
         <v>PASS</v>
       </c>
       <c r="H250">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="251">
@@ -7082,7 +7082,7 @@
         <v>PASS</v>
       </c>
       <c r="H251">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="252" xml:space="preserve">
@@ -7109,7 +7109,7 @@
         <v>PASS</v>
       </c>
       <c r="H252">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="253">
@@ -7135,7 +7135,7 @@
         <v>PASS</v>
       </c>
       <c r="H253">
-        <v>43</v>
+        <v>33</v>
       </c>
     </row>
     <row r="254">
@@ -7161,7 +7161,7 @@
         <v>PASS</v>
       </c>
       <c r="H254">
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="255">
@@ -7187,7 +7187,7 @@
         <v>PASS</v>
       </c>
       <c r="H255">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="256">
@@ -7213,7 +7213,7 @@
         <v>PASS</v>
       </c>
       <c r="H256">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="257">
@@ -7239,7 +7239,7 @@
         <v>PASS</v>
       </c>
       <c r="H257">
-        <v>15</v>
+        <v>43</v>
       </c>
     </row>
     <row r="258">
@@ -7265,7 +7265,7 @@
         <v>PASS</v>
       </c>
       <c r="H258">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="259">
@@ -7291,7 +7291,7 @@
         <v>PASS</v>
       </c>
       <c r="H259">
-        <v>32</v>
+        <v>50</v>
       </c>
     </row>
     <row r="260">
@@ -7317,7 +7317,7 @@
         <v>PASS</v>
       </c>
       <c r="H260">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="261">
@@ -7343,7 +7343,7 @@
         <v>PASS</v>
       </c>
       <c r="H261">
-        <v>16</v>
+        <v>39</v>
       </c>
     </row>
     <row r="262">
@@ -7369,7 +7369,7 @@
         <v>PASS</v>
       </c>
       <c r="H262">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="263">
@@ -7395,7 +7395,7 @@
         <v>PASS</v>
       </c>
       <c r="H263">
-        <v>33</v>
+        <v>46</v>
       </c>
     </row>
     <row r="264">
@@ -7421,7 +7421,7 @@
         <v>PASS</v>
       </c>
       <c r="H264">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="265">
@@ -7447,7 +7447,7 @@
         <v>PASS</v>
       </c>
       <c r="H265">
-        <v>17</v>
+        <v>38</v>
       </c>
     </row>
     <row r="266">
@@ -7473,7 +7473,7 @@
         <v>PASS</v>
       </c>
       <c r="H266">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="267">
@@ -7525,7 +7525,7 @@
         <v>PASS</v>
       </c>
       <c r="H268">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="269">
@@ -7551,7 +7551,7 @@
         <v>PASS</v>
       </c>
       <c r="H269">
-        <v>49</v>
+        <v>21</v>
       </c>
     </row>
     <row r="270">
@@ -7577,7 +7577,7 @@
         <v>PASS</v>
       </c>
       <c r="H270">
-        <v>36</v>
+        <v>48</v>
       </c>
     </row>
     <row r="271">
@@ -7603,7 +7603,7 @@
         <v>PASS</v>
       </c>
       <c r="H271">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="272" xml:space="preserve">
@@ -7630,7 +7630,7 @@
         <v>PASS</v>
       </c>
       <c r="H272">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="273">
@@ -7656,7 +7656,7 @@
         <v>PASS</v>
       </c>
       <c r="H273">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="274">
@@ -7682,7 +7682,7 @@
         <v>PASS</v>
       </c>
       <c r="H274">
-        <v>46</v>
+        <v>21</v>
       </c>
     </row>
     <row r="275">
@@ -7708,7 +7708,7 @@
         <v>PASS</v>
       </c>
       <c r="H275">
-        <v>39</v>
+        <v>15</v>
       </c>
     </row>
     <row r="276">
@@ -7734,7 +7734,7 @@
         <v>PASS</v>
       </c>
       <c r="H276">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="277">
@@ -7760,7 +7760,7 @@
         <v>PASS</v>
       </c>
       <c r="H277">
-        <v>42</v>
+        <v>20</v>
       </c>
     </row>
     <row r="278">
@@ -7786,7 +7786,7 @@
         <v>PASS</v>
       </c>
       <c r="H278">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="279">
@@ -7812,7 +7812,7 @@
         <v>PASS</v>
       </c>
       <c r="H279">
-        <v>15</v>
+        <v>26</v>
       </c>
     </row>
     <row r="280">
@@ -7838,7 +7838,7 @@
         <v>PASS</v>
       </c>
       <c r="H280">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="281">
@@ -7864,7 +7864,7 @@
         <v>PASS</v>
       </c>
       <c r="H281">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="282">
@@ -7916,7 +7916,7 @@
         <v>PASS</v>
       </c>
       <c r="H283">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="284">
@@ -7942,7 +7942,7 @@
         <v>PASS</v>
       </c>
       <c r="H284">
-        <v>44</v>
+        <v>30</v>
       </c>
     </row>
     <row r="285">
@@ -7968,7 +7968,7 @@
         <v>PASS</v>
       </c>
       <c r="H285">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="286">
@@ -7994,7 +7994,7 @@
         <v>PASS</v>
       </c>
       <c r="H286">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="287">
@@ -8020,7 +8020,7 @@
         <v>PASS</v>
       </c>
       <c r="H287">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="288">
@@ -8046,7 +8046,7 @@
         <v>PASS</v>
       </c>
       <c r="H288">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="289">
@@ -8072,7 +8072,7 @@
         <v>PASS</v>
       </c>
       <c r="H289">
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="290">
@@ -8098,7 +8098,7 @@
         <v>PASS</v>
       </c>
       <c r="H290">
-        <v>48</v>
+        <v>28</v>
       </c>
     </row>
     <row r="291">
@@ -8124,7 +8124,7 @@
         <v>PASS</v>
       </c>
       <c r="H291">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="292">
@@ -8150,7 +8150,7 @@
         <v>PASS</v>
       </c>
       <c r="H292">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="293">
@@ -8176,7 +8176,7 @@
         <v>PASS</v>
       </c>
       <c r="H293">
-        <v>30</v>
+        <v>45</v>
       </c>
     </row>
     <row r="294">
@@ -8202,7 +8202,7 @@
         <v>PASS</v>
       </c>
       <c r="H294">
-        <v>25</v>
+        <v>38</v>
       </c>
     </row>
     <row r="295">
@@ -8228,7 +8228,7 @@
         <v>PASS</v>
       </c>
       <c r="H295">
-        <v>41</v>
+        <v>31</v>
       </c>
     </row>
     <row r="296">
@@ -8254,7 +8254,7 @@
         <v>PASS</v>
       </c>
       <c r="H296">
-        <v>28</v>
+        <v>49</v>
       </c>
     </row>
     <row r="297">
@@ -8280,7 +8280,7 @@
         <v>PASS</v>
       </c>
       <c r="H297">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="298">
@@ -8306,7 +8306,7 @@
         <v>PASS</v>
       </c>
       <c r="H298">
-        <v>20</v>
+        <v>37</v>
       </c>
     </row>
     <row r="299">
@@ -8332,7 +8332,7 @@
         <v>PASS</v>
       </c>
       <c r="H299">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="300" xml:space="preserve">
@@ -8359,7 +8359,7 @@
         <v>PASS</v>
       </c>
       <c r="H300">
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
     <row r="301">
@@ -8385,7 +8385,7 @@
         <v>PASS</v>
       </c>
       <c r="H301">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(appium): clean silent exit & sync repository main branch
</commit_message>
<xml_diff>
--- a/appium-tests/Appium_E2E_Test_Report.xlsx
+++ b/appium-tests/Appium_E2E_Test_Report.xlsx
@@ -465,7 +465,7 @@
         <v>Execution Date &amp; Time</v>
       </c>
       <c r="B8" t="str">
-        <v>1/8/2026, 12:40:51 pm</v>
+        <v>5/8/2026, 1:10:06 pm</v>
       </c>
     </row>
     <row r="9">
@@ -586,7 +586,7 @@
         <v>PASS</v>
       </c>
       <c r="H2">
-        <v>42</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -613,7 +613,7 @@
         <v>PASS</v>
       </c>
       <c r="H3">
-        <v>47</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -639,7 +639,7 @@
         <v>PASS</v>
       </c>
       <c r="H4">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -665,7 +665,7 @@
         <v>PASS</v>
       </c>
       <c r="H5">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -691,7 +691,7 @@
         <v>PASS</v>
       </c>
       <c r="H6">
-        <v>18</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -718,7 +718,7 @@
         <v>PASS</v>
       </c>
       <c r="H7">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -771,7 +771,7 @@
         <v>PASS</v>
       </c>
       <c r="H9">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10">
@@ -797,7 +797,7 @@
         <v>PASS</v>
       </c>
       <c r="H10">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -824,7 +824,7 @@
         <v>PASS</v>
       </c>
       <c r="H11">
-        <v>51</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12">
@@ -850,7 +850,7 @@
         <v>PASS</v>
       </c>
       <c r="H12">
-        <v>32</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -876,7 +876,7 @@
         <v>PASS</v>
       </c>
       <c r="H13">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14">
@@ -902,7 +902,7 @@
         <v>PASS</v>
       </c>
       <c r="H14">
-        <v>16</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15">
@@ -928,7 +928,7 @@
         <v>PASS</v>
       </c>
       <c r="H15">
-        <v>48</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16">
@@ -954,7 +954,7 @@
         <v>PASS</v>
       </c>
       <c r="H16">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17">
@@ -980,7 +980,7 @@
         <v>PASS</v>
       </c>
       <c r="H17">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18">
@@ -1006,7 +1006,7 @@
         <v>PASS</v>
       </c>
       <c r="H18">
-        <v>51</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19">
@@ -1032,7 +1032,7 @@
         <v>PASS</v>
       </c>
       <c r="H19">
-        <v>23</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20">
@@ -1058,7 +1058,7 @@
         <v>PASS</v>
       </c>
       <c r="H20">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21">
@@ -1084,7 +1084,7 @@
         <v>PASS</v>
       </c>
       <c r="H21">
-        <v>29</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -1111,7 +1111,7 @@
         <v>PASS</v>
       </c>
       <c r="H22">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23">
@@ -1137,7 +1137,7 @@
         <v>PASS</v>
       </c>
       <c r="H23">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24">
@@ -1163,7 +1163,7 @@
         <v>PASS</v>
       </c>
       <c r="H24">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25">
@@ -1189,7 +1189,7 @@
         <v>PASS</v>
       </c>
       <c r="H25">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26">
@@ -1215,7 +1215,7 @@
         <v>PASS</v>
       </c>
       <c r="H26">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27">
@@ -1241,7 +1241,7 @@
         <v>PASS</v>
       </c>
       <c r="H27">
-        <v>47</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28">
@@ -1267,7 +1267,7 @@
         <v>PASS</v>
       </c>
       <c r="H28">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="29">
@@ -1293,7 +1293,7 @@
         <v>PASS</v>
       </c>
       <c r="H29">
-        <v>48</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30">
@@ -1319,7 +1319,7 @@
         <v>PASS</v>
       </c>
       <c r="H30">
-        <v>48</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31">
@@ -1345,7 +1345,7 @@
         <v>PASS</v>
       </c>
       <c r="H31">
-        <v>51</v>
+        <v>16</v>
       </c>
     </row>
     <row r="32">
@@ -1371,7 +1371,7 @@
         <v>PASS</v>
       </c>
       <c r="H32">
-        <v>45</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33">
@@ -1397,7 +1397,7 @@
         <v>PASS</v>
       </c>
       <c r="H33">
-        <v>37</v>
+        <v>51</v>
       </c>
     </row>
     <row r="34">
@@ -1423,7 +1423,7 @@
         <v>PASS</v>
       </c>
       <c r="H34">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35">
@@ -1449,7 +1449,7 @@
         <v>PASS</v>
       </c>
       <c r="H35">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36">
@@ -1475,7 +1475,7 @@
         <v>PASS</v>
       </c>
       <c r="H36">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="37">
@@ -1501,7 +1501,7 @@
         <v>PASS</v>
       </c>
       <c r="H37">
-        <v>40</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38">
@@ -1527,7 +1527,7 @@
         <v>PASS</v>
       </c>
       <c r="H38">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="39">
@@ -1553,7 +1553,7 @@
         <v>PASS</v>
       </c>
       <c r="H39">
-        <v>32</v>
+        <v>46</v>
       </c>
     </row>
     <row r="40">
@@ -1579,7 +1579,7 @@
         <v>PASS</v>
       </c>
       <c r="H40">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="41">
@@ -1605,7 +1605,7 @@
         <v>PASS</v>
       </c>
       <c r="H41">
-        <v>18</v>
+        <v>32</v>
       </c>
     </row>
     <row r="42">
@@ -1631,7 +1631,7 @@
         <v>PASS</v>
       </c>
       <c r="H42">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43">
@@ -1657,7 +1657,7 @@
         <v>PASS</v>
       </c>
       <c r="H43">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44">
@@ -1683,7 +1683,7 @@
         <v>PASS</v>
       </c>
       <c r="H44">
-        <v>40</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45">
@@ -1709,7 +1709,7 @@
         <v>PASS</v>
       </c>
       <c r="H45">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="46">
@@ -1735,7 +1735,7 @@
         <v>PASS</v>
       </c>
       <c r="H46">
-        <v>30</v>
+        <v>13</v>
       </c>
     </row>
     <row r="47">
@@ -1761,7 +1761,7 @@
         <v>PASS</v>
       </c>
       <c r="H47">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="48">
@@ -1787,7 +1787,7 @@
         <v>PASS</v>
       </c>
       <c r="H48">
-        <v>31</v>
+        <v>49</v>
       </c>
     </row>
     <row r="49">
@@ -1813,7 +1813,7 @@
         <v>PASS</v>
       </c>
       <c r="H49">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="50" xml:space="preserve">
@@ -1840,7 +1840,7 @@
         <v>PASS</v>
       </c>
       <c r="H50">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="51">
@@ -1866,7 +1866,7 @@
         <v>PASS</v>
       </c>
       <c r="H51">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="52">
@@ -1892,7 +1892,7 @@
         <v>PASS</v>
       </c>
       <c r="H52">
-        <v>47</v>
+        <v>19</v>
       </c>
     </row>
     <row r="53">
@@ -1918,7 +1918,7 @@
         <v>PASS</v>
       </c>
       <c r="H53">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="54">
@@ -1944,7 +1944,7 @@
         <v>PASS</v>
       </c>
       <c r="H54">
-        <v>27</v>
+        <v>19</v>
       </c>
     </row>
     <row r="55">
@@ -1970,7 +1970,7 @@
         <v>PASS</v>
       </c>
       <c r="H55">
-        <v>41</v>
+        <v>21</v>
       </c>
     </row>
     <row r="56">
@@ -1996,7 +1996,7 @@
         <v>PASS</v>
       </c>
       <c r="H56">
-        <v>45</v>
+        <v>31</v>
       </c>
     </row>
     <row r="57">
@@ -2022,7 +2022,7 @@
         <v>PASS</v>
       </c>
       <c r="H57">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="58">
@@ -2048,7 +2048,7 @@
         <v>PASS</v>
       </c>
       <c r="H58">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="59" xml:space="preserve">
@@ -2075,7 +2075,7 @@
         <v>PASS</v>
       </c>
       <c r="H59">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="60">
@@ -2101,7 +2101,7 @@
         <v>PASS</v>
       </c>
       <c r="H60">
-        <v>50</v>
+        <v>24</v>
       </c>
     </row>
     <row r="61">
@@ -2127,7 +2127,7 @@
         <v>PASS</v>
       </c>
       <c r="H61">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="62">
@@ -2153,7 +2153,7 @@
         <v>PASS</v>
       </c>
       <c r="H62">
-        <v>17</v>
+        <v>36</v>
       </c>
     </row>
     <row r="63">
@@ -2179,7 +2179,7 @@
         <v>PASS</v>
       </c>
       <c r="H63">
-        <v>17</v>
+        <v>32</v>
       </c>
     </row>
     <row r="64">
@@ -2205,7 +2205,7 @@
         <v>PASS</v>
       </c>
       <c r="H64">
-        <v>18</v>
+        <v>45</v>
       </c>
     </row>
     <row r="65">
@@ -2231,7 +2231,7 @@
         <v>PASS</v>
       </c>
       <c r="H65">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="66">
@@ -2257,7 +2257,7 @@
         <v>PASS</v>
       </c>
       <c r="H66">
-        <v>17</v>
+        <v>41</v>
       </c>
     </row>
     <row r="67">
@@ -2283,7 +2283,7 @@
         <v>PASS</v>
       </c>
       <c r="H67">
-        <v>24</v>
+        <v>45</v>
       </c>
     </row>
     <row r="68">
@@ -2309,7 +2309,7 @@
         <v>PASS</v>
       </c>
       <c r="H68">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="69">
@@ -2335,7 +2335,7 @@
         <v>PASS</v>
       </c>
       <c r="H69">
-        <v>43</v>
+        <v>27</v>
       </c>
     </row>
     <row r="70">
@@ -2361,7 +2361,7 @@
         <v>PASS</v>
       </c>
       <c r="H70">
-        <v>45</v>
+        <v>22</v>
       </c>
     </row>
     <row r="71">
@@ -2387,7 +2387,7 @@
         <v>PASS</v>
       </c>
       <c r="H71">
-        <v>51</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72">
@@ -2413,7 +2413,7 @@
         <v>PASS</v>
       </c>
       <c r="H72">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="73" xml:space="preserve">
@@ -2440,7 +2440,7 @@
         <v>PASS</v>
       </c>
       <c r="H73">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="74">
@@ -2466,7 +2466,7 @@
         <v>PASS</v>
       </c>
       <c r="H74">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="75">
@@ -2492,7 +2492,7 @@
         <v>PASS</v>
       </c>
       <c r="H75">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="76">
@@ -2518,7 +2518,7 @@
         <v>PASS</v>
       </c>
       <c r="H76">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="77">
@@ -2544,7 +2544,7 @@
         <v>PASS</v>
       </c>
       <c r="H77">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="78">
@@ -2570,7 +2570,7 @@
         <v>PASS</v>
       </c>
       <c r="H78">
-        <v>24</v>
+        <v>50</v>
       </c>
     </row>
     <row r="79">
@@ -2596,7 +2596,7 @@
         <v>PASS</v>
       </c>
       <c r="H79">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="80">
@@ -2622,7 +2622,7 @@
         <v>PASS</v>
       </c>
       <c r="H80">
-        <v>43</v>
+        <v>31</v>
       </c>
     </row>
     <row r="81">
@@ -2648,7 +2648,7 @@
         <v>PASS</v>
       </c>
       <c r="H81">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="82">
@@ -2674,7 +2674,7 @@
         <v>PASS</v>
       </c>
       <c r="H82">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="83">
@@ -2700,7 +2700,7 @@
         <v>PASS</v>
       </c>
       <c r="H83">
-        <v>14</v>
+        <v>39</v>
       </c>
     </row>
     <row r="84">
@@ -2726,7 +2726,7 @@
         <v>PASS</v>
       </c>
       <c r="H84">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="85">
@@ -2779,7 +2779,7 @@
         <v>PASS</v>
       </c>
       <c r="H86">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="87" xml:space="preserve">
@@ -2806,7 +2806,7 @@
         <v>PASS</v>
       </c>
       <c r="H87">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="88">
@@ -2832,7 +2832,7 @@
         <v>PASS</v>
       </c>
       <c r="H88">
-        <v>28</v>
+        <v>46</v>
       </c>
     </row>
     <row r="89">
@@ -2858,7 +2858,7 @@
         <v>PASS</v>
       </c>
       <c r="H89">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="90" xml:space="preserve">
@@ -2885,7 +2885,7 @@
         <v>PASS</v>
       </c>
       <c r="H90">
-        <v>45</v>
+        <v>16</v>
       </c>
     </row>
     <row r="91">
@@ -2911,7 +2911,7 @@
         <v>PASS</v>
       </c>
       <c r="H91">
-        <v>18</v>
+        <v>39</v>
       </c>
     </row>
     <row r="92">
@@ -2937,7 +2937,7 @@
         <v>PASS</v>
       </c>
       <c r="H92">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="93">
@@ -2963,7 +2963,7 @@
         <v>PASS</v>
       </c>
       <c r="H93">
-        <v>34</v>
+        <v>14</v>
       </c>
     </row>
     <row r="94">
@@ -2989,7 +2989,7 @@
         <v>PASS</v>
       </c>
       <c r="H94">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="95">
@@ -3015,7 +3015,7 @@
         <v>PASS</v>
       </c>
       <c r="H95">
-        <v>22</v>
+        <v>36</v>
       </c>
     </row>
     <row r="96">
@@ -3041,7 +3041,7 @@
         <v>PASS</v>
       </c>
       <c r="H96">
-        <v>32</v>
+        <v>51</v>
       </c>
     </row>
     <row r="97">
@@ -3067,7 +3067,7 @@
         <v>PASS</v>
       </c>
       <c r="H97">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="98">
@@ -3093,7 +3093,7 @@
         <v>PASS</v>
       </c>
       <c r="H98">
-        <v>13</v>
+        <v>34</v>
       </c>
     </row>
     <row r="99">
@@ -3119,7 +3119,7 @@
         <v>PASS</v>
       </c>
       <c r="H99">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="100">
@@ -3145,7 +3145,7 @@
         <v>PASS</v>
       </c>
       <c r="H100">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="101">
@@ -3171,7 +3171,7 @@
         <v>PASS</v>
       </c>
       <c r="H101">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="102">
@@ -3197,7 +3197,7 @@
         <v>PASS</v>
       </c>
       <c r="H102">
-        <v>37</v>
+        <v>18</v>
       </c>
     </row>
     <row r="103">
@@ -3223,7 +3223,7 @@
         <v>PASS</v>
       </c>
       <c r="H103">
-        <v>30</v>
+        <v>17</v>
       </c>
     </row>
     <row r="104">
@@ -3275,7 +3275,7 @@
         <v>PASS</v>
       </c>
       <c r="H105">
-        <v>35</v>
+        <v>14</v>
       </c>
     </row>
     <row r="106">
@@ -3301,7 +3301,7 @@
         <v>PASS</v>
       </c>
       <c r="H106">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="107">
@@ -3327,7 +3327,7 @@
         <v>PASS</v>
       </c>
       <c r="H107">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="108">
@@ -3353,7 +3353,7 @@
         <v>PASS</v>
       </c>
       <c r="H108">
-        <v>50</v>
+        <v>30</v>
       </c>
     </row>
     <row r="109">
@@ -3379,7 +3379,7 @@
         <v>PASS</v>
       </c>
       <c r="H109">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="110">
@@ -3405,7 +3405,7 @@
         <v>PASS</v>
       </c>
       <c r="H110">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
     <row r="111">
@@ -3431,7 +3431,7 @@
         <v>PASS</v>
       </c>
       <c r="H111">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="112">
@@ -3457,7 +3457,7 @@
         <v>PASS</v>
       </c>
       <c r="H112">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="113">
@@ -3483,7 +3483,7 @@
         <v>PASS</v>
       </c>
       <c r="H113">
-        <v>23</v>
+        <v>38</v>
       </c>
     </row>
     <row r="114">
@@ -3509,7 +3509,7 @@
         <v>PASS</v>
       </c>
       <c r="H114">
-        <v>23</v>
+        <v>51</v>
       </c>
     </row>
     <row r="115">
@@ -3535,7 +3535,7 @@
         <v>PASS</v>
       </c>
       <c r="H115">
-        <v>47</v>
+        <v>16</v>
       </c>
     </row>
     <row r="116">
@@ -3561,7 +3561,7 @@
         <v>PASS</v>
       </c>
       <c r="H116">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="117">
@@ -3587,7 +3587,7 @@
         <v>PASS</v>
       </c>
       <c r="H117">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="118">
@@ -3613,7 +3613,7 @@
         <v>PASS</v>
       </c>
       <c r="H118">
-        <v>18</v>
+        <v>31</v>
       </c>
     </row>
     <row r="119">
@@ -3639,7 +3639,7 @@
         <v>PASS</v>
       </c>
       <c r="H119">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="120">
@@ -3665,7 +3665,7 @@
         <v>PASS</v>
       </c>
       <c r="H120">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="121">
@@ -3691,7 +3691,7 @@
         <v>PASS</v>
       </c>
       <c r="H121">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="122">
@@ -3717,7 +3717,7 @@
         <v>PASS</v>
       </c>
       <c r="H122">
-        <v>37</v>
+        <v>20</v>
       </c>
     </row>
     <row r="123">
@@ -3743,7 +3743,7 @@
         <v>PASS</v>
       </c>
       <c r="H123">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="124">
@@ -3769,7 +3769,7 @@
         <v>PASS</v>
       </c>
       <c r="H124">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="125">
@@ -3795,7 +3795,7 @@
         <v>PASS</v>
       </c>
       <c r="H125">
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
     <row r="126">
@@ -3821,7 +3821,7 @@
         <v>PASS</v>
       </c>
       <c r="H126">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127">
@@ -3847,7 +3847,7 @@
         <v>PASS</v>
       </c>
       <c r="H127">
-        <v>28</v>
+        <v>39</v>
       </c>
     </row>
     <row r="128">
@@ -3873,7 +3873,7 @@
         <v>PASS</v>
       </c>
       <c r="H128">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="129" xml:space="preserve">
@@ -3900,7 +3900,7 @@
         <v>PASS</v>
       </c>
       <c r="H129">
-        <v>50</v>
+        <v>27</v>
       </c>
     </row>
     <row r="130">
@@ -3952,7 +3952,7 @@
         <v>PASS</v>
       </c>
       <c r="H131">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="132">
@@ -3978,7 +3978,7 @@
         <v>PASS</v>
       </c>
       <c r="H132">
-        <v>41</v>
+        <v>26</v>
       </c>
     </row>
     <row r="133">
@@ -4004,7 +4004,7 @@
         <v>PASS</v>
       </c>
       <c r="H133">
-        <v>47</v>
+        <v>27</v>
       </c>
     </row>
     <row r="134" xml:space="preserve">
@@ -4031,7 +4031,7 @@
         <v>PASS</v>
       </c>
       <c r="H134">
-        <v>28</v>
+        <v>42</v>
       </c>
     </row>
     <row r="135">
@@ -4057,7 +4057,7 @@
         <v>PASS</v>
       </c>
       <c r="H135">
-        <v>31</v>
+        <v>46</v>
       </c>
     </row>
     <row r="136">
@@ -4083,7 +4083,7 @@
         <v>PASS</v>
       </c>
       <c r="H136">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="137">
@@ -4109,7 +4109,7 @@
         <v>PASS</v>
       </c>
       <c r="H137">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="138">
@@ -4135,7 +4135,7 @@
         <v>PASS</v>
       </c>
       <c r="H138">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="139">
@@ -4161,7 +4161,7 @@
         <v>PASS</v>
       </c>
       <c r="H139">
-        <v>32</v>
+        <v>46</v>
       </c>
     </row>
     <row r="140">
@@ -4187,7 +4187,7 @@
         <v>PASS</v>
       </c>
       <c r="H140">
-        <v>20</v>
+        <v>42</v>
       </c>
     </row>
     <row r="141">
@@ -4213,7 +4213,7 @@
         <v>PASS</v>
       </c>
       <c r="H141">
-        <v>12</v>
+        <v>41</v>
       </c>
     </row>
     <row r="142">
@@ -4239,7 +4239,7 @@
         <v>PASS</v>
       </c>
       <c r="H142">
-        <v>39</v>
+        <v>21</v>
       </c>
     </row>
     <row r="143">
@@ -4265,7 +4265,7 @@
         <v>PASS</v>
       </c>
       <c r="H143">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="144">
@@ -4291,7 +4291,7 @@
         <v>PASS</v>
       </c>
       <c r="H144">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="145">
@@ -4317,7 +4317,7 @@
         <v>PASS</v>
       </c>
       <c r="H145">
-        <v>33</v>
+        <v>15</v>
       </c>
     </row>
     <row r="146">
@@ -4343,7 +4343,7 @@
         <v>PASS</v>
       </c>
       <c r="H146">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="147">
@@ -4369,7 +4369,7 @@
         <v>PASS</v>
       </c>
       <c r="H147">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="148">
@@ -4395,7 +4395,7 @@
         <v>PASS</v>
       </c>
       <c r="H148">
-        <v>23</v>
+        <v>42</v>
       </c>
     </row>
     <row r="149">
@@ -4421,7 +4421,7 @@
         <v>PASS</v>
       </c>
       <c r="H149">
-        <v>15</v>
+        <v>45</v>
       </c>
     </row>
     <row r="150">
@@ -4447,7 +4447,7 @@
         <v>PASS</v>
       </c>
       <c r="H150">
-        <v>46</v>
+        <v>19</v>
       </c>
     </row>
     <row r="151">
@@ -4473,7 +4473,7 @@
         <v>PASS</v>
       </c>
       <c r="H151">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="152">
@@ -4499,7 +4499,7 @@
         <v>PASS</v>
       </c>
       <c r="H152">
-        <v>30</v>
+        <v>23</v>
       </c>
     </row>
     <row r="153">
@@ -4525,7 +4525,7 @@
         <v>PASS</v>
       </c>
       <c r="H153">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="154">
@@ -4551,7 +4551,7 @@
         <v>PASS</v>
       </c>
       <c r="H154">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="155">
@@ -4577,7 +4577,7 @@
         <v>PASS</v>
       </c>
       <c r="H155">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="156">
@@ -4603,7 +4603,7 @@
         <v>PASS</v>
       </c>
       <c r="H156">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="157">
@@ -4629,7 +4629,7 @@
         <v>PASS</v>
       </c>
       <c r="H157">
-        <v>45</v>
+        <v>21</v>
       </c>
     </row>
     <row r="158">
@@ -4655,7 +4655,7 @@
         <v>PASS</v>
       </c>
       <c r="H158">
-        <v>31</v>
+        <v>43</v>
       </c>
     </row>
     <row r="159">
@@ -4681,7 +4681,7 @@
         <v>PASS</v>
       </c>
       <c r="H159">
-        <v>23</v>
+        <v>50</v>
       </c>
     </row>
     <row r="160">
@@ -4707,7 +4707,7 @@
         <v>PASS</v>
       </c>
       <c r="H160">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="161">
@@ -4733,7 +4733,7 @@
         <v>PASS</v>
       </c>
       <c r="H161">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="162">
@@ -4759,7 +4759,7 @@
         <v>PASS</v>
       </c>
       <c r="H162">
-        <v>37</v>
+        <v>50</v>
       </c>
     </row>
     <row r="163">
@@ -4785,7 +4785,7 @@
         <v>PASS</v>
       </c>
       <c r="H163">
-        <v>50</v>
+        <v>35</v>
       </c>
     </row>
     <row r="164">
@@ -4811,7 +4811,7 @@
         <v>PASS</v>
       </c>
       <c r="H164">
-        <v>28</v>
+        <v>13</v>
       </c>
     </row>
     <row r="165">
@@ -4837,7 +4837,7 @@
         <v>PASS</v>
       </c>
       <c r="H165">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="166">
@@ -4863,7 +4863,7 @@
         <v>PASS</v>
       </c>
       <c r="H166">
-        <v>48</v>
+        <v>32</v>
       </c>
     </row>
     <row r="167">
@@ -4889,7 +4889,7 @@
         <v>PASS</v>
       </c>
       <c r="H167">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="168">
@@ -4915,7 +4915,7 @@
         <v>PASS</v>
       </c>
       <c r="H168">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="169">
@@ -4941,7 +4941,7 @@
         <v>PASS</v>
       </c>
       <c r="H169">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="170">
@@ -4967,7 +4967,7 @@
         <v>PASS</v>
       </c>
       <c r="H170">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="171">
@@ -4993,7 +4993,7 @@
         <v>PASS</v>
       </c>
       <c r="H171">
-        <v>26</v>
+        <v>19</v>
       </c>
     </row>
     <row r="172">
@@ -5019,7 +5019,7 @@
         <v>PASS</v>
       </c>
       <c r="H172">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="173">
@@ -5045,7 +5045,7 @@
         <v>PASS</v>
       </c>
       <c r="H173">
-        <v>16</v>
+        <v>42</v>
       </c>
     </row>
     <row r="174">
@@ -5071,7 +5071,7 @@
         <v>PASS</v>
       </c>
       <c r="H174">
-        <v>17</v>
+        <v>39</v>
       </c>
     </row>
     <row r="175">
@@ -5097,7 +5097,7 @@
         <v>PASS</v>
       </c>
       <c r="H175">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="176" xml:space="preserve">
@@ -5124,7 +5124,7 @@
         <v>PASS</v>
       </c>
       <c r="H176">
-        <v>15</v>
+        <v>45</v>
       </c>
     </row>
     <row r="177">
@@ -5150,7 +5150,7 @@
         <v>PASS</v>
       </c>
       <c r="H177">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="178">
@@ -5176,7 +5176,7 @@
         <v>PASS</v>
       </c>
       <c r="H178">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="179">
@@ -5202,7 +5202,7 @@
         <v>PASS</v>
       </c>
       <c r="H179">
-        <v>44</v>
+        <v>20</v>
       </c>
     </row>
     <row r="180">
@@ -5228,7 +5228,7 @@
         <v>PASS</v>
       </c>
       <c r="H180">
-        <v>34</v>
+        <v>21</v>
       </c>
     </row>
     <row r="181">
@@ -5254,7 +5254,7 @@
         <v>PASS</v>
       </c>
       <c r="H181">
-        <v>32</v>
+        <v>47</v>
       </c>
     </row>
     <row r="182">
@@ -5280,7 +5280,7 @@
         <v>PASS</v>
       </c>
       <c r="H182">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="183">
@@ -5306,7 +5306,7 @@
         <v>PASS</v>
       </c>
       <c r="H183">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="184">
@@ -5332,7 +5332,7 @@
         <v>PASS</v>
       </c>
       <c r="H184">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="185">
@@ -5358,7 +5358,7 @@
         <v>PASS</v>
       </c>
       <c r="H185">
-        <v>16</v>
+        <v>43</v>
       </c>
     </row>
     <row r="186" xml:space="preserve">
@@ -5385,7 +5385,7 @@
         <v>PASS</v>
       </c>
       <c r="H186">
-        <v>12</v>
+        <v>37</v>
       </c>
     </row>
     <row r="187" xml:space="preserve">
@@ -5412,7 +5412,7 @@
         <v>PASS</v>
       </c>
       <c r="H187">
-        <v>42</v>
+        <v>22</v>
       </c>
     </row>
     <row r="188">
@@ -5438,7 +5438,7 @@
         <v>PASS</v>
       </c>
       <c r="H188">
-        <v>14</v>
+        <v>42</v>
       </c>
     </row>
     <row r="189">
@@ -5464,7 +5464,7 @@
         <v>PASS</v>
       </c>
       <c r="H189">
-        <v>20</v>
+        <v>38</v>
       </c>
     </row>
     <row r="190">
@@ -5490,7 +5490,7 @@
         <v>PASS</v>
       </c>
       <c r="H190">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="191">
@@ -5516,7 +5516,7 @@
         <v>PASS</v>
       </c>
       <c r="H191">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="192">
@@ -5568,7 +5568,7 @@
         <v>PASS</v>
       </c>
       <c r="H193">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="194">
@@ -5620,7 +5620,7 @@
         <v>PASS</v>
       </c>
       <c r="H195">
-        <v>44</v>
+        <v>19</v>
       </c>
     </row>
     <row r="196">
@@ -5646,7 +5646,7 @@
         <v>PASS</v>
       </c>
       <c r="H196">
-        <v>24</v>
+        <v>45</v>
       </c>
     </row>
     <row r="197">
@@ -5672,7 +5672,7 @@
         <v>PASS</v>
       </c>
       <c r="H197">
-        <v>12</v>
+        <v>44</v>
       </c>
     </row>
     <row r="198">
@@ -5698,7 +5698,7 @@
         <v>PASS</v>
       </c>
       <c r="H198">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="199">
@@ -5724,7 +5724,7 @@
         <v>PASS</v>
       </c>
       <c r="H199">
-        <v>17</v>
+        <v>35</v>
       </c>
     </row>
     <row r="200">
@@ -5750,7 +5750,7 @@
         <v>PASS</v>
       </c>
       <c r="H200">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="201">
@@ -5776,7 +5776,7 @@
         <v>PASS</v>
       </c>
       <c r="H201">
-        <v>25</v>
+        <v>37</v>
       </c>
     </row>
     <row r="202">
@@ -5802,7 +5802,7 @@
         <v>PASS</v>
       </c>
       <c r="H202">
-        <v>13</v>
+        <v>30</v>
       </c>
     </row>
     <row r="203">
@@ -5828,7 +5828,7 @@
         <v>PASS</v>
       </c>
       <c r="H203">
-        <v>17</v>
+        <v>49</v>
       </c>
     </row>
     <row r="204">
@@ -5854,7 +5854,7 @@
         <v>PASS</v>
       </c>
       <c r="H204">
-        <v>35</v>
+        <v>14</v>
       </c>
     </row>
     <row r="205">
@@ -5880,7 +5880,7 @@
         <v>PASS</v>
       </c>
       <c r="H205">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="206">
@@ -5906,7 +5906,7 @@
         <v>PASS</v>
       </c>
       <c r="H206">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="207">
@@ -5932,7 +5932,7 @@
         <v>PASS</v>
       </c>
       <c r="H207">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="208">
@@ -5958,7 +5958,7 @@
         <v>PASS</v>
       </c>
       <c r="H208">
-        <v>36</v>
+        <v>15</v>
       </c>
     </row>
     <row r="209">
@@ -5984,7 +5984,7 @@
         <v>PASS</v>
       </c>
       <c r="H209">
-        <v>27</v>
+        <v>50</v>
       </c>
     </row>
     <row r="210">
@@ -6010,7 +6010,7 @@
         <v>PASS</v>
       </c>
       <c r="H210">
-        <v>45</v>
+        <v>18</v>
       </c>
     </row>
     <row r="211" xml:space="preserve">
@@ -6037,7 +6037,7 @@
         <v>PASS</v>
       </c>
       <c r="H211">
-        <v>42</v>
+        <v>24</v>
       </c>
     </row>
     <row r="212">
@@ -6063,7 +6063,7 @@
         <v>PASS</v>
       </c>
       <c r="H212">
-        <v>12</v>
+        <v>22</v>
       </c>
     </row>
     <row r="213">
@@ -6089,7 +6089,7 @@
         <v>PASS</v>
       </c>
       <c r="H213">
-        <v>17</v>
+        <v>31</v>
       </c>
     </row>
     <row r="214">
@@ -6115,7 +6115,7 @@
         <v>PASS</v>
       </c>
       <c r="H214">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="215">
@@ -6141,7 +6141,7 @@
         <v>PASS</v>
       </c>
       <c r="H215">
-        <v>14</v>
+        <v>48</v>
       </c>
     </row>
     <row r="216">
@@ -6167,7 +6167,7 @@
         <v>PASS</v>
       </c>
       <c r="H216">
-        <v>42</v>
+        <v>24</v>
       </c>
     </row>
     <row r="217">
@@ -6193,7 +6193,7 @@
         <v>PASS</v>
       </c>
       <c r="H217">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="218">
@@ -6219,7 +6219,7 @@
         <v>PASS</v>
       </c>
       <c r="H218">
-        <v>45</v>
+        <v>22</v>
       </c>
     </row>
     <row r="219">
@@ -6245,7 +6245,7 @@
         <v>PASS</v>
       </c>
       <c r="H219">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="220">
@@ -6271,7 +6271,7 @@
         <v>PASS</v>
       </c>
       <c r="H220">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
     <row r="221">
@@ -6297,7 +6297,7 @@
         <v>PASS</v>
       </c>
       <c r="H221">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="222">
@@ -6323,7 +6323,7 @@
         <v>PASS</v>
       </c>
       <c r="H222">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="223">
@@ -6349,7 +6349,7 @@
         <v>PASS</v>
       </c>
       <c r="H223">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="224">
@@ -6375,7 +6375,7 @@
         <v>PASS</v>
       </c>
       <c r="H224">
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="225">
@@ -6401,7 +6401,7 @@
         <v>PASS</v>
       </c>
       <c r="H225">
-        <v>36</v>
+        <v>15</v>
       </c>
     </row>
     <row r="226">
@@ -6427,7 +6427,7 @@
         <v>PASS</v>
       </c>
       <c r="H226">
-        <v>12</v>
+        <v>31</v>
       </c>
     </row>
     <row r="227">
@@ -6453,7 +6453,7 @@
         <v>PASS</v>
       </c>
       <c r="H227">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="228">
@@ -6479,7 +6479,7 @@
         <v>PASS</v>
       </c>
       <c r="H228">
-        <v>14</v>
+        <v>32</v>
       </c>
     </row>
     <row r="229">
@@ -6505,7 +6505,7 @@
         <v>PASS</v>
       </c>
       <c r="H229">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="230">
@@ -6531,7 +6531,7 @@
         <v>PASS</v>
       </c>
       <c r="H230">
-        <v>23</v>
+        <v>47</v>
       </c>
     </row>
     <row r="231">
@@ -6557,7 +6557,7 @@
         <v>PASS</v>
       </c>
       <c r="H231">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="232">
@@ -6583,7 +6583,7 @@
         <v>PASS</v>
       </c>
       <c r="H232">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="233">
@@ -6609,7 +6609,7 @@
         <v>PASS</v>
       </c>
       <c r="H233">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="234">
@@ -6635,7 +6635,7 @@
         <v>PASS</v>
       </c>
       <c r="H234">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="235">
@@ -6661,7 +6661,7 @@
         <v>PASS</v>
       </c>
       <c r="H235">
-        <v>48</v>
+        <v>17</v>
       </c>
     </row>
     <row r="236">
@@ -6687,7 +6687,7 @@
         <v>PASS</v>
       </c>
       <c r="H236">
-        <v>45</v>
+        <v>22</v>
       </c>
     </row>
     <row r="237">
@@ -6713,7 +6713,7 @@
         <v>PASS</v>
       </c>
       <c r="H237">
-        <v>29</v>
+        <v>45</v>
       </c>
     </row>
     <row r="238" xml:space="preserve">
@@ -6740,7 +6740,7 @@
         <v>PASS</v>
       </c>
       <c r="H238">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="239">
@@ -6766,7 +6766,7 @@
         <v>PASS</v>
       </c>
       <c r="H239">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="240">
@@ -6792,7 +6792,7 @@
         <v>PASS</v>
       </c>
       <c r="H240">
-        <v>49</v>
+        <v>32</v>
       </c>
     </row>
     <row r="241">
@@ -6818,7 +6818,7 @@
         <v>PASS</v>
       </c>
       <c r="H241">
-        <v>35</v>
+        <v>49</v>
       </c>
     </row>
     <row r="242">
@@ -6844,7 +6844,7 @@
         <v>PASS</v>
       </c>
       <c r="H242">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="243" xml:space="preserve">
@@ -6871,7 +6871,7 @@
         <v>PASS</v>
       </c>
       <c r="H243">
-        <v>50</v>
+        <v>28</v>
       </c>
     </row>
     <row r="244">
@@ -6897,7 +6897,7 @@
         <v>PASS</v>
       </c>
       <c r="H244">
-        <v>26</v>
+        <v>44</v>
       </c>
     </row>
     <row r="245">
@@ -6923,7 +6923,7 @@
         <v>PASS</v>
       </c>
       <c r="H245">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="246">
@@ -6949,7 +6949,7 @@
         <v>PASS</v>
       </c>
       <c r="H246">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="247">
@@ -6975,7 +6975,7 @@
         <v>PASS</v>
       </c>
       <c r="H247">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="248" xml:space="preserve">
@@ -7030,7 +7030,7 @@
         <v>PASS</v>
       </c>
       <c r="H249">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="250">
@@ -7056,7 +7056,7 @@
         <v>PASS</v>
       </c>
       <c r="H250">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="251">
@@ -7082,7 +7082,7 @@
         <v>PASS</v>
       </c>
       <c r="H251">
-        <v>26</v>
+        <v>46</v>
       </c>
     </row>
     <row r="252" xml:space="preserve">
@@ -7109,7 +7109,7 @@
         <v>PASS</v>
       </c>
       <c r="H252">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="253">
@@ -7135,7 +7135,7 @@
         <v>PASS</v>
       </c>
       <c r="H253">
-        <v>33</v>
+        <v>16</v>
       </c>
     </row>
     <row r="254">
@@ -7161,7 +7161,7 @@
         <v>PASS</v>
       </c>
       <c r="H254">
-        <v>28</v>
+        <v>15</v>
       </c>
     </row>
     <row r="255">
@@ -7187,7 +7187,7 @@
         <v>PASS</v>
       </c>
       <c r="H255">
-        <v>22</v>
+        <v>51</v>
       </c>
     </row>
     <row r="256">
@@ -7213,7 +7213,7 @@
         <v>PASS</v>
       </c>
       <c r="H256">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="257">
@@ -7239,7 +7239,7 @@
         <v>PASS</v>
       </c>
       <c r="H257">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="258">
@@ -7265,7 +7265,7 @@
         <v>PASS</v>
       </c>
       <c r="H258">
-        <v>12</v>
+        <v>42</v>
       </c>
     </row>
     <row r="259">
@@ -7291,7 +7291,7 @@
         <v>PASS</v>
       </c>
       <c r="H259">
-        <v>50</v>
+        <v>16</v>
       </c>
     </row>
     <row r="260">
@@ -7317,7 +7317,7 @@
         <v>PASS</v>
       </c>
       <c r="H260">
-        <v>49</v>
+        <v>25</v>
       </c>
     </row>
     <row r="261">
@@ -7343,7 +7343,7 @@
         <v>PASS</v>
       </c>
       <c r="H261">
-        <v>39</v>
+        <v>15</v>
       </c>
     </row>
     <row r="262">
@@ -7369,7 +7369,7 @@
         <v>PASS</v>
       </c>
       <c r="H262">
-        <v>26</v>
+        <v>40</v>
       </c>
     </row>
     <row r="263">
@@ -7395,7 +7395,7 @@
         <v>PASS</v>
       </c>
       <c r="H263">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="264">
@@ -7421,7 +7421,7 @@
         <v>PASS</v>
       </c>
       <c r="H264">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="265">
@@ -7447,7 +7447,7 @@
         <v>PASS</v>
       </c>
       <c r="H265">
-        <v>38</v>
+        <v>26</v>
       </c>
     </row>
     <row r="266">
@@ -7473,7 +7473,7 @@
         <v>PASS</v>
       </c>
       <c r="H266">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="267">
@@ -7499,7 +7499,7 @@
         <v>PASS</v>
       </c>
       <c r="H267">
-        <v>22</v>
+        <v>41</v>
       </c>
     </row>
     <row r="268">
@@ -7525,7 +7525,7 @@
         <v>PASS</v>
       </c>
       <c r="H268">
-        <v>43</v>
+        <v>24</v>
       </c>
     </row>
     <row r="269">
@@ -7551,7 +7551,7 @@
         <v>PASS</v>
       </c>
       <c r="H269">
-        <v>21</v>
+        <v>40</v>
       </c>
     </row>
     <row r="270">
@@ -7577,7 +7577,7 @@
         <v>PASS</v>
       </c>
       <c r="H270">
-        <v>48</v>
+        <v>15</v>
       </c>
     </row>
     <row r="271">
@@ -7603,7 +7603,7 @@
         <v>PASS</v>
       </c>
       <c r="H271">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="272" xml:space="preserve">
@@ -7630,7 +7630,7 @@
         <v>PASS</v>
       </c>
       <c r="H272">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="273">
@@ -7656,7 +7656,7 @@
         <v>PASS</v>
       </c>
       <c r="H273">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="274">
@@ -7682,7 +7682,7 @@
         <v>PASS</v>
       </c>
       <c r="H274">
-        <v>21</v>
+        <v>50</v>
       </c>
     </row>
     <row r="275">
@@ -7708,7 +7708,7 @@
         <v>PASS</v>
       </c>
       <c r="H275">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="276">
@@ -7734,7 +7734,7 @@
         <v>PASS</v>
       </c>
       <c r="H276">
-        <v>22</v>
+        <v>49</v>
       </c>
     </row>
     <row r="277">
@@ -7760,7 +7760,7 @@
         <v>PASS</v>
       </c>
       <c r="H277">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="278">
@@ -7786,7 +7786,7 @@
         <v>PASS</v>
       </c>
       <c r="H278">
-        <v>12</v>
+        <v>35</v>
       </c>
     </row>
     <row r="279">
@@ -7812,7 +7812,7 @@
         <v>PASS</v>
       </c>
       <c r="H279">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="280">
@@ -7838,7 +7838,7 @@
         <v>PASS</v>
       </c>
       <c r="H280">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
     <row r="281">
@@ -7864,7 +7864,7 @@
         <v>PASS</v>
       </c>
       <c r="H281">
-        <v>21</v>
+        <v>37</v>
       </c>
     </row>
     <row r="282">
@@ -7890,7 +7890,7 @@
         <v>PASS</v>
       </c>
       <c r="H282">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="283">
@@ -7916,7 +7916,7 @@
         <v>PASS</v>
       </c>
       <c r="H283">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="284">
@@ -7942,7 +7942,7 @@
         <v>PASS</v>
       </c>
       <c r="H284">
-        <v>30</v>
+        <v>42</v>
       </c>
     </row>
     <row r="285">
@@ -7968,7 +7968,7 @@
         <v>PASS</v>
       </c>
       <c r="H285">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="286">
@@ -7994,7 +7994,7 @@
         <v>PASS</v>
       </c>
       <c r="H286">
-        <v>22</v>
+        <v>43</v>
       </c>
     </row>
     <row r="287">
@@ -8020,7 +8020,7 @@
         <v>PASS</v>
       </c>
       <c r="H287">
-        <v>37</v>
+        <v>18</v>
       </c>
     </row>
     <row r="288">
@@ -8046,7 +8046,7 @@
         <v>PASS</v>
       </c>
       <c r="H288">
-        <v>32</v>
+        <v>22</v>
       </c>
     </row>
     <row r="289">
@@ -8072,7 +8072,7 @@
         <v>PASS</v>
       </c>
       <c r="H289">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="290">
@@ -8098,7 +8098,7 @@
         <v>PASS</v>
       </c>
       <c r="H290">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="291">
@@ -8124,7 +8124,7 @@
         <v>PASS</v>
       </c>
       <c r="H291">
-        <v>40</v>
+        <v>26</v>
       </c>
     </row>
     <row r="292">
@@ -8150,7 +8150,7 @@
         <v>PASS</v>
       </c>
       <c r="H292">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="293">
@@ -8176,7 +8176,7 @@
         <v>PASS</v>
       </c>
       <c r="H293">
-        <v>45</v>
+        <v>22</v>
       </c>
     </row>
     <row r="294">
@@ -8202,7 +8202,7 @@
         <v>PASS</v>
       </c>
       <c r="H294">
-        <v>38</v>
+        <v>31</v>
       </c>
     </row>
     <row r="295">
@@ -8228,7 +8228,7 @@
         <v>PASS</v>
       </c>
       <c r="H295">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="296">
@@ -8254,7 +8254,7 @@
         <v>PASS</v>
       </c>
       <c r="H296">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="297">
@@ -8280,7 +8280,7 @@
         <v>PASS</v>
       </c>
       <c r="H297">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="298">
@@ -8306,7 +8306,7 @@
         <v>PASS</v>
       </c>
       <c r="H298">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
     <row r="299">
@@ -8332,7 +8332,7 @@
         <v>PASS</v>
       </c>
       <c r="H299">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="300" xml:space="preserve">
@@ -8359,7 +8359,7 @@
         <v>PASS</v>
       </c>
       <c r="H300">
-        <v>27</v>
+        <v>41</v>
       </c>
     </row>
     <row r="301">
@@ -8385,7 +8385,7 @@
         <v>PASS</v>
       </c>
       <c r="H301">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: Appium 300 mobile E2E test suite report Excel artifact
</commit_message>
<xml_diff>
--- a/appium-tests/Appium_E2E_Test_Report.xlsx
+++ b/appium-tests/Appium_E2E_Test_Report.xlsx
@@ -465,7 +465,7 @@
         <v>Execution Date &amp; Time</v>
       </c>
       <c r="B8" t="str">
-        <v>5/8/2026, 1:10:06 pm</v>
+        <v>7/8/2026, 11:13:23 am</v>
       </c>
     </row>
     <row r="9">
@@ -586,7 +586,7 @@
         <v>PASS</v>
       </c>
       <c r="H2">
-        <v>51</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -613,7 +613,7 @@
         <v>PASS</v>
       </c>
       <c r="H3">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
@@ -639,7 +639,7 @@
         <v>PASS</v>
       </c>
       <c r="H4">
-        <v>38</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -665,7 +665,7 @@
         <v>PASS</v>
       </c>
       <c r="H5">
-        <v>27</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6">
@@ -691,7 +691,7 @@
         <v>PASS</v>
       </c>
       <c r="H6">
-        <v>33</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -718,7 +718,7 @@
         <v>PASS</v>
       </c>
       <c r="H7">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -744,7 +744,7 @@
         <v>PASS</v>
       </c>
       <c r="H8">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -771,7 +771,7 @@
         <v>PASS</v>
       </c>
       <c r="H9">
-        <v>36</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -797,7 +797,7 @@
         <v>PASS</v>
       </c>
       <c r="H10">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -824,7 +824,7 @@
         <v>PASS</v>
       </c>
       <c r="H11">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12">
@@ -850,7 +850,7 @@
         <v>PASS</v>
       </c>
       <c r="H12">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -876,7 +876,7 @@
         <v>PASS</v>
       </c>
       <c r="H13">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14">
@@ -902,7 +902,7 @@
         <v>PASS</v>
       </c>
       <c r="H14">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -928,7 +928,7 @@
         <v>PASS</v>
       </c>
       <c r="H15">
-        <v>41</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16">
@@ -954,7 +954,7 @@
         <v>PASS</v>
       </c>
       <c r="H16">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17">
@@ -980,7 +980,7 @@
         <v>PASS</v>
       </c>
       <c r="H17">
-        <v>42</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18">
@@ -1006,7 +1006,7 @@
         <v>PASS</v>
       </c>
       <c r="H18">
-        <v>26</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19">
@@ -1032,7 +1032,7 @@
         <v>PASS</v>
       </c>
       <c r="H19">
-        <v>42</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20">
@@ -1058,7 +1058,7 @@
         <v>PASS</v>
       </c>
       <c r="H20">
-        <v>45</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21">
@@ -1084,7 +1084,7 @@
         <v>PASS</v>
       </c>
       <c r="H21">
-        <v>15</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -1111,7 +1111,7 @@
         <v>PASS</v>
       </c>
       <c r="H22">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23">
@@ -1137,7 +1137,7 @@
         <v>PASS</v>
       </c>
       <c r="H23">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24">
@@ -1163,7 +1163,7 @@
         <v>PASS</v>
       </c>
       <c r="H24">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25">
@@ -1189,7 +1189,7 @@
         <v>PASS</v>
       </c>
       <c r="H25">
-        <v>42</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26">
@@ -1215,7 +1215,7 @@
         <v>PASS</v>
       </c>
       <c r="H26">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27">
@@ -1241,7 +1241,7 @@
         <v>PASS</v>
       </c>
       <c r="H27">
-        <v>29</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28">
@@ -1267,7 +1267,7 @@
         <v>PASS</v>
       </c>
       <c r="H28">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="29">
@@ -1293,7 +1293,7 @@
         <v>PASS</v>
       </c>
       <c r="H29">
-        <v>30</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30">
@@ -1319,7 +1319,7 @@
         <v>PASS</v>
       </c>
       <c r="H30">
-        <v>21</v>
+        <v>38</v>
       </c>
     </row>
     <row r="31">
@@ -1345,7 +1345,7 @@
         <v>PASS</v>
       </c>
       <c r="H31">
-        <v>16</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32">
@@ -1371,7 +1371,7 @@
         <v>PASS</v>
       </c>
       <c r="H32">
-        <v>14</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33">
@@ -1397,7 +1397,7 @@
         <v>PASS</v>
       </c>
       <c r="H33">
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34">
@@ -1423,7 +1423,7 @@
         <v>PASS</v>
       </c>
       <c r="H34">
-        <v>23</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35">
@@ -1449,7 +1449,7 @@
         <v>PASS</v>
       </c>
       <c r="H35">
-        <v>30</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36">
@@ -1475,7 +1475,7 @@
         <v>PASS</v>
       </c>
       <c r="H36">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="37">
@@ -1501,7 +1501,7 @@
         <v>PASS</v>
       </c>
       <c r="H37">
-        <v>26</v>
+        <v>38</v>
       </c>
     </row>
     <row r="38">
@@ -1527,7 +1527,7 @@
         <v>PASS</v>
       </c>
       <c r="H38">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="39">
@@ -1553,7 +1553,7 @@
         <v>PASS</v>
       </c>
       <c r="H39">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40">
@@ -1579,7 +1579,7 @@
         <v>PASS</v>
       </c>
       <c r="H40">
-        <v>28</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41">
@@ -1605,7 +1605,7 @@
         <v>PASS</v>
       </c>
       <c r="H41">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="42">
@@ -1631,7 +1631,7 @@
         <v>PASS</v>
       </c>
       <c r="H42">
-        <v>41</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43">
@@ -1657,7 +1657,7 @@
         <v>PASS</v>
       </c>
       <c r="H43">
-        <v>31</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44">
@@ -1683,7 +1683,7 @@
         <v>PASS</v>
       </c>
       <c r="H44">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="45">
@@ -1709,7 +1709,7 @@
         <v>PASS</v>
       </c>
       <c r="H45">
-        <v>34</v>
+        <v>24</v>
       </c>
     </row>
     <row r="46">
@@ -1735,7 +1735,7 @@
         <v>PASS</v>
       </c>
       <c r="H46">
-        <v>13</v>
+        <v>47</v>
       </c>
     </row>
     <row r="47">
@@ -1787,7 +1787,7 @@
         <v>PASS</v>
       </c>
       <c r="H48">
-        <v>49</v>
+        <v>21</v>
       </c>
     </row>
     <row r="49">
@@ -1813,7 +1813,7 @@
         <v>PASS</v>
       </c>
       <c r="H49">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50" xml:space="preserve">
@@ -1840,7 +1840,7 @@
         <v>PASS</v>
       </c>
       <c r="H50">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51">
@@ -1866,7 +1866,7 @@
         <v>PASS</v>
       </c>
       <c r="H51">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52">
@@ -1892,7 +1892,7 @@
         <v>PASS</v>
       </c>
       <c r="H52">
-        <v>19</v>
+        <v>43</v>
       </c>
     </row>
     <row r="53">
@@ -1918,7 +1918,7 @@
         <v>PASS</v>
       </c>
       <c r="H53">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="54">
@@ -1944,7 +1944,7 @@
         <v>PASS</v>
       </c>
       <c r="H54">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="55">
@@ -1970,7 +1970,7 @@
         <v>PASS</v>
       </c>
       <c r="H55">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="56">
@@ -1996,7 +1996,7 @@
         <v>PASS</v>
       </c>
       <c r="H56">
-        <v>31</v>
+        <v>41</v>
       </c>
     </row>
     <row r="57">
@@ -2022,7 +2022,7 @@
         <v>PASS</v>
       </c>
       <c r="H57">
-        <v>31</v>
+        <v>17</v>
       </c>
     </row>
     <row r="58">
@@ -2048,7 +2048,7 @@
         <v>PASS</v>
       </c>
       <c r="H58">
-        <v>15</v>
+        <v>26</v>
       </c>
     </row>
     <row r="59" xml:space="preserve">
@@ -2075,7 +2075,7 @@
         <v>PASS</v>
       </c>
       <c r="H59">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="60">
@@ -2101,7 +2101,7 @@
         <v>PASS</v>
       </c>
       <c r="H60">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="61">
@@ -2127,7 +2127,7 @@
         <v>PASS</v>
       </c>
       <c r="H61">
-        <v>31</v>
+        <v>50</v>
       </c>
     </row>
     <row r="62">
@@ -2153,7 +2153,7 @@
         <v>PASS</v>
       </c>
       <c r="H62">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="63">
@@ -2179,7 +2179,7 @@
         <v>PASS</v>
       </c>
       <c r="H63">
-        <v>32</v>
+        <v>13</v>
       </c>
     </row>
     <row r="64">
@@ -2205,7 +2205,7 @@
         <v>PASS</v>
       </c>
       <c r="H64">
-        <v>45</v>
+        <v>15</v>
       </c>
     </row>
     <row r="65">
@@ -2231,7 +2231,7 @@
         <v>PASS</v>
       </c>
       <c r="H65">
-        <v>24</v>
+        <v>39</v>
       </c>
     </row>
     <row r="66">
@@ -2257,7 +2257,7 @@
         <v>PASS</v>
       </c>
       <c r="H66">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="67">
@@ -2283,7 +2283,7 @@
         <v>PASS</v>
       </c>
       <c r="H67">
-        <v>45</v>
+        <v>23</v>
       </c>
     </row>
     <row r="68">
@@ -2309,7 +2309,7 @@
         <v>PASS</v>
       </c>
       <c r="H68">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="69">
@@ -2335,7 +2335,7 @@
         <v>PASS</v>
       </c>
       <c r="H69">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="70">
@@ -2361,7 +2361,7 @@
         <v>PASS</v>
       </c>
       <c r="H70">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="71">
@@ -2387,7 +2387,7 @@
         <v>PASS</v>
       </c>
       <c r="H71">
-        <v>34</v>
+        <v>25</v>
       </c>
     </row>
     <row r="72">
@@ -2413,7 +2413,7 @@
         <v>PASS</v>
       </c>
       <c r="H72">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="73" xml:space="preserve">
@@ -2440,7 +2440,7 @@
         <v>PASS</v>
       </c>
       <c r="H73">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="74">
@@ -2466,7 +2466,7 @@
         <v>PASS</v>
       </c>
       <c r="H74">
-        <v>30</v>
+        <v>18</v>
       </c>
     </row>
     <row r="75">
@@ -2492,7 +2492,7 @@
         <v>PASS</v>
       </c>
       <c r="H75">
-        <v>19</v>
+        <v>33</v>
       </c>
     </row>
     <row r="76">
@@ -2518,7 +2518,7 @@
         <v>PASS</v>
       </c>
       <c r="H76">
-        <v>29</v>
+        <v>14</v>
       </c>
     </row>
     <row r="77">
@@ -2544,7 +2544,7 @@
         <v>PASS</v>
       </c>
       <c r="H77">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="78">
@@ -2570,7 +2570,7 @@
         <v>PASS</v>
       </c>
       <c r="H78">
-        <v>50</v>
+        <v>21</v>
       </c>
     </row>
     <row r="79">
@@ -2596,7 +2596,7 @@
         <v>PASS</v>
       </c>
       <c r="H79">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="80">
@@ -2622,7 +2622,7 @@
         <v>PASS</v>
       </c>
       <c r="H80">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="81">
@@ -2674,7 +2674,7 @@
         <v>PASS</v>
       </c>
       <c r="H82">
-        <v>28</v>
+        <v>46</v>
       </c>
     </row>
     <row r="83">
@@ -2700,7 +2700,7 @@
         <v>PASS</v>
       </c>
       <c r="H83">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="84">
@@ -2726,7 +2726,7 @@
         <v>PASS</v>
       </c>
       <c r="H84">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="85">
@@ -2752,7 +2752,7 @@
         <v>PASS</v>
       </c>
       <c r="H85">
-        <v>45</v>
+        <v>22</v>
       </c>
     </row>
     <row r="86" xml:space="preserve">
@@ -2779,7 +2779,7 @@
         <v>PASS</v>
       </c>
       <c r="H86">
-        <v>38</v>
+        <v>49</v>
       </c>
     </row>
     <row r="87" xml:space="preserve">
@@ -2806,7 +2806,7 @@
         <v>PASS</v>
       </c>
       <c r="H87">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="88">
@@ -2832,7 +2832,7 @@
         <v>PASS</v>
       </c>
       <c r="H88">
-        <v>46</v>
+        <v>18</v>
       </c>
     </row>
     <row r="89">
@@ -2858,7 +2858,7 @@
         <v>PASS</v>
       </c>
       <c r="H89">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="90" xml:space="preserve">
@@ -2885,7 +2885,7 @@
         <v>PASS</v>
       </c>
       <c r="H90">
-        <v>16</v>
+        <v>32</v>
       </c>
     </row>
     <row r="91">
@@ -2911,7 +2911,7 @@
         <v>PASS</v>
       </c>
       <c r="H91">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="92">
@@ -2937,7 +2937,7 @@
         <v>PASS</v>
       </c>
       <c r="H92">
-        <v>12</v>
+        <v>27</v>
       </c>
     </row>
     <row r="93">
@@ -2963,7 +2963,7 @@
         <v>PASS</v>
       </c>
       <c r="H93">
-        <v>14</v>
+        <v>29</v>
       </c>
     </row>
     <row r="94">
@@ -2989,7 +2989,7 @@
         <v>PASS</v>
       </c>
       <c r="H94">
-        <v>51</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95">
@@ -3015,7 +3015,7 @@
         <v>PASS</v>
       </c>
       <c r="H95">
-        <v>36</v>
+        <v>15</v>
       </c>
     </row>
     <row r="96">
@@ -3041,7 +3041,7 @@
         <v>PASS</v>
       </c>
       <c r="H96">
-        <v>51</v>
+        <v>23</v>
       </c>
     </row>
     <row r="97">
@@ -3067,7 +3067,7 @@
         <v>PASS</v>
       </c>
       <c r="H97">
-        <v>43</v>
+        <v>33</v>
       </c>
     </row>
     <row r="98">
@@ -3093,7 +3093,7 @@
         <v>PASS</v>
       </c>
       <c r="H98">
-        <v>34</v>
+        <v>25</v>
       </c>
     </row>
     <row r="99">
@@ -3119,7 +3119,7 @@
         <v>PASS</v>
       </c>
       <c r="H99">
-        <v>24</v>
+        <v>48</v>
       </c>
     </row>
     <row r="100">
@@ -3145,7 +3145,7 @@
         <v>PASS</v>
       </c>
       <c r="H100">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="101">
@@ -3171,7 +3171,7 @@
         <v>PASS</v>
       </c>
       <c r="H101">
-        <v>33</v>
+        <v>15</v>
       </c>
     </row>
     <row r="102">
@@ -3197,7 +3197,7 @@
         <v>PASS</v>
       </c>
       <c r="H102">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="103">
@@ -3223,7 +3223,7 @@
         <v>PASS</v>
       </c>
       <c r="H103">
-        <v>17</v>
+        <v>49</v>
       </c>
     </row>
     <row r="104">
@@ -3249,7 +3249,7 @@
         <v>PASS</v>
       </c>
       <c r="H104">
-        <v>51</v>
+        <v>31</v>
       </c>
     </row>
     <row r="105">
@@ -3275,7 +3275,7 @@
         <v>PASS</v>
       </c>
       <c r="H105">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="106">
@@ -3301,7 +3301,7 @@
         <v>PASS</v>
       </c>
       <c r="H106">
-        <v>35</v>
+        <v>18</v>
       </c>
     </row>
     <row r="107">
@@ -3327,7 +3327,7 @@
         <v>PASS</v>
       </c>
       <c r="H107">
-        <v>23</v>
+        <v>40</v>
       </c>
     </row>
     <row r="108">
@@ -3353,7 +3353,7 @@
         <v>PASS</v>
       </c>
       <c r="H108">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="109">
@@ -3379,7 +3379,7 @@
         <v>PASS</v>
       </c>
       <c r="H109">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="110">
@@ -3405,7 +3405,7 @@
         <v>PASS</v>
       </c>
       <c r="H110">
-        <v>27</v>
+        <v>46</v>
       </c>
     </row>
     <row r="111">
@@ -3431,7 +3431,7 @@
         <v>PASS</v>
       </c>
       <c r="H111">
-        <v>19</v>
+        <v>51</v>
       </c>
     </row>
     <row r="112">
@@ -3457,7 +3457,7 @@
         <v>PASS</v>
       </c>
       <c r="H112">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="113">
@@ -3483,7 +3483,7 @@
         <v>PASS</v>
       </c>
       <c r="H113">
-        <v>38</v>
+        <v>12</v>
       </c>
     </row>
     <row r="114">
@@ -3509,7 +3509,7 @@
         <v>PASS</v>
       </c>
       <c r="H114">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="115">
@@ -3535,7 +3535,7 @@
         <v>PASS</v>
       </c>
       <c r="H115">
-        <v>16</v>
+        <v>41</v>
       </c>
     </row>
     <row r="116">
@@ -3561,7 +3561,7 @@
         <v>PASS</v>
       </c>
       <c r="H116">
-        <v>43</v>
+        <v>14</v>
       </c>
     </row>
     <row r="117">
@@ -3587,7 +3587,7 @@
         <v>PASS</v>
       </c>
       <c r="H117">
-        <v>42</v>
+        <v>18</v>
       </c>
     </row>
     <row r="118">
@@ -3639,7 +3639,7 @@
         <v>PASS</v>
       </c>
       <c r="H119">
-        <v>45</v>
+        <v>12</v>
       </c>
     </row>
     <row r="120">
@@ -3665,7 +3665,7 @@
         <v>PASS</v>
       </c>
       <c r="H120">
-        <v>49</v>
+        <v>18</v>
       </c>
     </row>
     <row r="121">
@@ -3691,7 +3691,7 @@
         <v>PASS</v>
       </c>
       <c r="H121">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="122">
@@ -3717,7 +3717,7 @@
         <v>PASS</v>
       </c>
       <c r="H122">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="123">
@@ -3743,7 +3743,7 @@
         <v>PASS</v>
       </c>
       <c r="H123">
-        <v>35</v>
+        <v>21</v>
       </c>
     </row>
     <row r="124">
@@ -3769,7 +3769,7 @@
         <v>PASS</v>
       </c>
       <c r="H124">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="125">
@@ -3795,7 +3795,7 @@
         <v>PASS</v>
       </c>
       <c r="H125">
-        <v>27</v>
+        <v>38</v>
       </c>
     </row>
     <row r="126">
@@ -3821,7 +3821,7 @@
         <v>PASS</v>
       </c>
       <c r="H126">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="127">
@@ -3847,7 +3847,7 @@
         <v>PASS</v>
       </c>
       <c r="H127">
-        <v>39</v>
+        <v>22</v>
       </c>
     </row>
     <row r="128">
@@ -3873,7 +3873,7 @@
         <v>PASS</v>
       </c>
       <c r="H128">
-        <v>30</v>
+        <v>48</v>
       </c>
     </row>
     <row r="129" xml:space="preserve">
@@ -3900,7 +3900,7 @@
         <v>PASS</v>
       </c>
       <c r="H129">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="130">
@@ -3926,7 +3926,7 @@
         <v>PASS</v>
       </c>
       <c r="H130">
-        <v>49</v>
+        <v>28</v>
       </c>
     </row>
     <row r="131">
@@ -3952,7 +3952,7 @@
         <v>PASS</v>
       </c>
       <c r="H131">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="132">
@@ -3978,7 +3978,7 @@
         <v>PASS</v>
       </c>
       <c r="H132">
-        <v>26</v>
+        <v>46</v>
       </c>
     </row>
     <row r="133">
@@ -4004,7 +4004,7 @@
         <v>PASS</v>
       </c>
       <c r="H133">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="134" xml:space="preserve">
@@ -4031,7 +4031,7 @@
         <v>PASS</v>
       </c>
       <c r="H134">
-        <v>42</v>
+        <v>13</v>
       </c>
     </row>
     <row r="135">
@@ -4057,7 +4057,7 @@
         <v>PASS</v>
       </c>
       <c r="H135">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="136">
@@ -4083,7 +4083,7 @@
         <v>PASS</v>
       </c>
       <c r="H136">
-        <v>40</v>
+        <v>14</v>
       </c>
     </row>
     <row r="137">
@@ -4109,7 +4109,7 @@
         <v>PASS</v>
       </c>
       <c r="H137">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="138">
@@ -4135,7 +4135,7 @@
         <v>PASS</v>
       </c>
       <c r="H138">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="139">
@@ -4161,7 +4161,7 @@
         <v>PASS</v>
       </c>
       <c r="H139">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="140">
@@ -4187,7 +4187,7 @@
         <v>PASS</v>
       </c>
       <c r="H140">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="141">
@@ -4213,7 +4213,7 @@
         <v>PASS</v>
       </c>
       <c r="H141">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="142">
@@ -4239,7 +4239,7 @@
         <v>PASS</v>
       </c>
       <c r="H142">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="143">
@@ -4265,7 +4265,7 @@
         <v>PASS</v>
       </c>
       <c r="H143">
-        <v>18</v>
+        <v>40</v>
       </c>
     </row>
     <row r="144">
@@ -4291,7 +4291,7 @@
         <v>PASS</v>
       </c>
       <c r="H144">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="145">
@@ -4317,7 +4317,7 @@
         <v>PASS</v>
       </c>
       <c r="H145">
-        <v>15</v>
+        <v>43</v>
       </c>
     </row>
     <row r="146">
@@ -4343,7 +4343,7 @@
         <v>PASS</v>
       </c>
       <c r="H146">
-        <v>50</v>
+        <v>30</v>
       </c>
     </row>
     <row r="147">
@@ -4369,7 +4369,7 @@
         <v>PASS</v>
       </c>
       <c r="H147">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="148">
@@ -4395,7 +4395,7 @@
         <v>PASS</v>
       </c>
       <c r="H148">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="149">
@@ -4421,7 +4421,7 @@
         <v>PASS</v>
       </c>
       <c r="H149">
-        <v>45</v>
+        <v>14</v>
       </c>
     </row>
     <row r="150">
@@ -4447,7 +4447,7 @@
         <v>PASS</v>
       </c>
       <c r="H150">
-        <v>19</v>
+        <v>47</v>
       </c>
     </row>
     <row r="151">
@@ -4473,7 +4473,7 @@
         <v>PASS</v>
       </c>
       <c r="H151">
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="152">
@@ -4499,7 +4499,7 @@
         <v>PASS</v>
       </c>
       <c r="H152">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="153">
@@ -4525,7 +4525,7 @@
         <v>PASS</v>
       </c>
       <c r="H153">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="154">
@@ -4551,7 +4551,7 @@
         <v>PASS</v>
       </c>
       <c r="H154">
-        <v>21</v>
+        <v>39</v>
       </c>
     </row>
     <row r="155">
@@ -4577,7 +4577,7 @@
         <v>PASS</v>
       </c>
       <c r="H155">
-        <v>37</v>
+        <v>12</v>
       </c>
     </row>
     <row r="156">
@@ -4603,7 +4603,7 @@
         <v>PASS</v>
       </c>
       <c r="H156">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="157">
@@ -4629,7 +4629,7 @@
         <v>PASS</v>
       </c>
       <c r="H157">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="158">
@@ -4655,7 +4655,7 @@
         <v>PASS</v>
       </c>
       <c r="H158">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="159">
@@ -4681,7 +4681,7 @@
         <v>PASS</v>
       </c>
       <c r="H159">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="160">
@@ -4707,7 +4707,7 @@
         <v>PASS</v>
       </c>
       <c r="H160">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="161">
@@ -4733,7 +4733,7 @@
         <v>PASS</v>
       </c>
       <c r="H161">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="162">
@@ -4759,7 +4759,7 @@
         <v>PASS</v>
       </c>
       <c r="H162">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="163">
@@ -4785,7 +4785,7 @@
         <v>PASS</v>
       </c>
       <c r="H163">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="164">
@@ -4837,7 +4837,7 @@
         <v>PASS</v>
       </c>
       <c r="H165">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="166">
@@ -4863,7 +4863,7 @@
         <v>PASS</v>
       </c>
       <c r="H166">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
     <row r="167">
@@ -4889,7 +4889,7 @@
         <v>PASS</v>
       </c>
       <c r="H167">
-        <v>38</v>
+        <v>24</v>
       </c>
     </row>
     <row r="168">
@@ -4915,7 +4915,7 @@
         <v>PASS</v>
       </c>
       <c r="H168">
-        <v>25</v>
+        <v>43</v>
       </c>
     </row>
     <row r="169">
@@ -4941,7 +4941,7 @@
         <v>PASS</v>
       </c>
       <c r="H169">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="170">
@@ -4967,7 +4967,7 @@
         <v>PASS</v>
       </c>
       <c r="H170">
-        <v>21</v>
+        <v>50</v>
       </c>
     </row>
     <row r="171">
@@ -4993,7 +4993,7 @@
         <v>PASS</v>
       </c>
       <c r="H171">
-        <v>19</v>
+        <v>42</v>
       </c>
     </row>
     <row r="172">
@@ -5019,7 +5019,7 @@
         <v>PASS</v>
       </c>
       <c r="H172">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="173">
@@ -5045,7 +5045,7 @@
         <v>PASS</v>
       </c>
       <c r="H173">
-        <v>42</v>
+        <v>14</v>
       </c>
     </row>
     <row r="174">
@@ -5071,7 +5071,7 @@
         <v>PASS</v>
       </c>
       <c r="H174">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="175">
@@ -5097,7 +5097,7 @@
         <v>PASS</v>
       </c>
       <c r="H175">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="176" xml:space="preserve">
@@ -5124,7 +5124,7 @@
         <v>PASS</v>
       </c>
       <c r="H176">
-        <v>45</v>
+        <v>32</v>
       </c>
     </row>
     <row r="177">
@@ -5150,7 +5150,7 @@
         <v>PASS</v>
       </c>
       <c r="H177">
-        <v>20</v>
+        <v>46</v>
       </c>
     </row>
     <row r="178">
@@ -5176,7 +5176,7 @@
         <v>PASS</v>
       </c>
       <c r="H178">
-        <v>17</v>
+        <v>36</v>
       </c>
     </row>
     <row r="179">
@@ -5202,7 +5202,7 @@
         <v>PASS</v>
       </c>
       <c r="H179">
-        <v>20</v>
+        <v>41</v>
       </c>
     </row>
     <row r="180">
@@ -5228,7 +5228,7 @@
         <v>PASS</v>
       </c>
       <c r="H180">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="181">
@@ -5254,7 +5254,7 @@
         <v>PASS</v>
       </c>
       <c r="H181">
-        <v>47</v>
+        <v>25</v>
       </c>
     </row>
     <row r="182">
@@ -5280,7 +5280,7 @@
         <v>PASS</v>
       </c>
       <c r="H182">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="183">
@@ -5306,7 +5306,7 @@
         <v>PASS</v>
       </c>
       <c r="H183">
-        <v>20</v>
+        <v>31</v>
       </c>
     </row>
     <row r="184">
@@ -5332,7 +5332,7 @@
         <v>PASS</v>
       </c>
       <c r="H184">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="185">
@@ -5358,7 +5358,7 @@
         <v>PASS</v>
       </c>
       <c r="H185">
-        <v>43</v>
+        <v>29</v>
       </c>
     </row>
     <row r="186" xml:space="preserve">
@@ -5385,7 +5385,7 @@
         <v>PASS</v>
       </c>
       <c r="H186">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="187" xml:space="preserve">
@@ -5412,7 +5412,7 @@
         <v>PASS</v>
       </c>
       <c r="H187">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="188">
@@ -5438,7 +5438,7 @@
         <v>PASS</v>
       </c>
       <c r="H188">
-        <v>42</v>
+        <v>28</v>
       </c>
     </row>
     <row r="189">
@@ -5464,7 +5464,7 @@
         <v>PASS</v>
       </c>
       <c r="H189">
-        <v>38</v>
+        <v>12</v>
       </c>
     </row>
     <row r="190">
@@ -5490,7 +5490,7 @@
         <v>PASS</v>
       </c>
       <c r="H190">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="191">
@@ -5516,7 +5516,7 @@
         <v>PASS</v>
       </c>
       <c r="H191">
-        <v>19</v>
+        <v>42</v>
       </c>
     </row>
     <row r="192">
@@ -5542,7 +5542,7 @@
         <v>PASS</v>
       </c>
       <c r="H192">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="193">
@@ -5568,7 +5568,7 @@
         <v>PASS</v>
       </c>
       <c r="H193">
-        <v>13</v>
+        <v>27</v>
       </c>
     </row>
     <row r="194">
@@ -5594,7 +5594,7 @@
         <v>PASS</v>
       </c>
       <c r="H194">
-        <v>34</v>
+        <v>50</v>
       </c>
     </row>
     <row r="195">
@@ -5620,7 +5620,7 @@
         <v>PASS</v>
       </c>
       <c r="H195">
-        <v>19</v>
+        <v>51</v>
       </c>
     </row>
     <row r="196">
@@ -5646,7 +5646,7 @@
         <v>PASS</v>
       </c>
       <c r="H196">
-        <v>45</v>
+        <v>19</v>
       </c>
     </row>
     <row r="197">
@@ -5672,7 +5672,7 @@
         <v>PASS</v>
       </c>
       <c r="H197">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="198">
@@ -5698,7 +5698,7 @@
         <v>PASS</v>
       </c>
       <c r="H198">
-        <v>26</v>
+        <v>41</v>
       </c>
     </row>
     <row r="199">
@@ -5724,7 +5724,7 @@
         <v>PASS</v>
       </c>
       <c r="H199">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="200">
@@ -5750,7 +5750,7 @@
         <v>PASS</v>
       </c>
       <c r="H200">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="201">
@@ -5776,7 +5776,7 @@
         <v>PASS</v>
       </c>
       <c r="H201">
-        <v>37</v>
+        <v>12</v>
       </c>
     </row>
     <row r="202">
@@ -5802,7 +5802,7 @@
         <v>PASS</v>
       </c>
       <c r="H202">
-        <v>30</v>
+        <v>13</v>
       </c>
     </row>
     <row r="203">
@@ -5828,7 +5828,7 @@
         <v>PASS</v>
       </c>
       <c r="H203">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="204">
@@ -5854,7 +5854,7 @@
         <v>PASS</v>
       </c>
       <c r="H204">
-        <v>14</v>
+        <v>39</v>
       </c>
     </row>
     <row r="205">
@@ -5880,7 +5880,7 @@
         <v>PASS</v>
       </c>
       <c r="H205">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="206">
@@ -5906,7 +5906,7 @@
         <v>PASS</v>
       </c>
       <c r="H206">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="207">
@@ -5932,7 +5932,7 @@
         <v>PASS</v>
       </c>
       <c r="H207">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="208">
@@ -5958,7 +5958,7 @@
         <v>PASS</v>
       </c>
       <c r="H208">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="209">
@@ -5984,7 +5984,7 @@
         <v>PASS</v>
       </c>
       <c r="H209">
-        <v>50</v>
+        <v>37</v>
       </c>
     </row>
     <row r="210">
@@ -6010,7 +6010,7 @@
         <v>PASS</v>
       </c>
       <c r="H210">
-        <v>18</v>
+        <v>33</v>
       </c>
     </row>
     <row r="211" xml:space="preserve">
@@ -6037,7 +6037,7 @@
         <v>PASS</v>
       </c>
       <c r="H211">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="212">
@@ -6089,7 +6089,7 @@
         <v>PASS</v>
       </c>
       <c r="H213">
-        <v>31</v>
+        <v>42</v>
       </c>
     </row>
     <row r="214">
@@ -6115,7 +6115,7 @@
         <v>PASS</v>
       </c>
       <c r="H214">
-        <v>14</v>
+        <v>49</v>
       </c>
     </row>
     <row r="215">
@@ -6141,7 +6141,7 @@
         <v>PASS</v>
       </c>
       <c r="H215">
-        <v>48</v>
+        <v>14</v>
       </c>
     </row>
     <row r="216">
@@ -6167,7 +6167,7 @@
         <v>PASS</v>
       </c>
       <c r="H216">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="217">
@@ -6193,7 +6193,7 @@
         <v>PASS</v>
       </c>
       <c r="H217">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="218">
@@ -6219,7 +6219,7 @@
         <v>PASS</v>
       </c>
       <c r="H218">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="219">
@@ -6245,7 +6245,7 @@
         <v>PASS</v>
       </c>
       <c r="H219">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="220">
@@ -6271,7 +6271,7 @@
         <v>PASS</v>
       </c>
       <c r="H220">
-        <v>50</v>
+        <v>14</v>
       </c>
     </row>
     <row r="221">
@@ -6297,7 +6297,7 @@
         <v>PASS</v>
       </c>
       <c r="H221">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="222">
@@ -6323,7 +6323,7 @@
         <v>PASS</v>
       </c>
       <c r="H222">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="223">
@@ -6349,7 +6349,7 @@
         <v>PASS</v>
       </c>
       <c r="H223">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="224">
@@ -6375,7 +6375,7 @@
         <v>PASS</v>
       </c>
       <c r="H224">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="225">
@@ -6401,7 +6401,7 @@
         <v>PASS</v>
       </c>
       <c r="H225">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="226">
@@ -6427,7 +6427,7 @@
         <v>PASS</v>
       </c>
       <c r="H226">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="227">
@@ -6453,7 +6453,7 @@
         <v>PASS</v>
       </c>
       <c r="H227">
-        <v>27</v>
+        <v>41</v>
       </c>
     </row>
     <row r="228">
@@ -6505,7 +6505,7 @@
         <v>PASS</v>
       </c>
       <c r="H229">
-        <v>18</v>
+        <v>29</v>
       </c>
     </row>
     <row r="230">
@@ -6531,7 +6531,7 @@
         <v>PASS</v>
       </c>
       <c r="H230">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="231">
@@ -6557,7 +6557,7 @@
         <v>PASS</v>
       </c>
       <c r="H231">
-        <v>24</v>
+        <v>31</v>
       </c>
     </row>
     <row r="232">
@@ -6583,7 +6583,7 @@
         <v>PASS</v>
       </c>
       <c r="H232">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="233">
@@ -6609,7 +6609,7 @@
         <v>PASS</v>
       </c>
       <c r="H233">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="234">
@@ -6635,7 +6635,7 @@
         <v>PASS</v>
       </c>
       <c r="H234">
-        <v>50</v>
+        <v>13</v>
       </c>
     </row>
     <row r="235">
@@ -6661,7 +6661,7 @@
         <v>PASS</v>
       </c>
       <c r="H235">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="236">
@@ -6687,7 +6687,7 @@
         <v>PASS</v>
       </c>
       <c r="H236">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="237">
@@ -6713,7 +6713,7 @@
         <v>PASS</v>
       </c>
       <c r="H237">
-        <v>45</v>
+        <v>25</v>
       </c>
     </row>
     <row r="238" xml:space="preserve">
@@ -6740,7 +6740,7 @@
         <v>PASS</v>
       </c>
       <c r="H238">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="239">
@@ -6766,7 +6766,7 @@
         <v>PASS</v>
       </c>
       <c r="H239">
-        <v>31</v>
+        <v>50</v>
       </c>
     </row>
     <row r="240">
@@ -6792,7 +6792,7 @@
         <v>PASS</v>
       </c>
       <c r="H240">
-        <v>32</v>
+        <v>13</v>
       </c>
     </row>
     <row r="241">
@@ -6818,7 +6818,7 @@
         <v>PASS</v>
       </c>
       <c r="H241">
-        <v>49</v>
+        <v>20</v>
       </c>
     </row>
     <row r="242">
@@ -6844,7 +6844,7 @@
         <v>PASS</v>
       </c>
       <c r="H242">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="243" xml:space="preserve">
@@ -6871,7 +6871,7 @@
         <v>PASS</v>
       </c>
       <c r="H243">
-        <v>28</v>
+        <v>18</v>
       </c>
     </row>
     <row r="244">
@@ -6897,7 +6897,7 @@
         <v>PASS</v>
       </c>
       <c r="H244">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="245">
@@ -6923,7 +6923,7 @@
         <v>PASS</v>
       </c>
       <c r="H245">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="246">
@@ -6949,7 +6949,7 @@
         <v>PASS</v>
       </c>
       <c r="H246">
-        <v>20</v>
+        <v>34</v>
       </c>
     </row>
     <row r="247">
@@ -6975,7 +6975,7 @@
         <v>PASS</v>
       </c>
       <c r="H247">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="248" xml:space="preserve">
@@ -7003,7 +7003,7 @@
         <v>PASS</v>
       </c>
       <c r="H248">
-        <v>24</v>
+        <v>39</v>
       </c>
     </row>
     <row r="249" xml:space="preserve">
@@ -7056,7 +7056,7 @@
         <v>PASS</v>
       </c>
       <c r="H250">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="251">
@@ -7082,7 +7082,7 @@
         <v>PASS</v>
       </c>
       <c r="H251">
-        <v>46</v>
+        <v>13</v>
       </c>
     </row>
     <row r="252" xml:space="preserve">
@@ -7109,7 +7109,7 @@
         <v>PASS</v>
       </c>
       <c r="H252">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="253">
@@ -7135,7 +7135,7 @@
         <v>PASS</v>
       </c>
       <c r="H253">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="254">
@@ -7161,7 +7161,7 @@
         <v>PASS</v>
       </c>
       <c r="H254">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="255">
@@ -7187,7 +7187,7 @@
         <v>PASS</v>
       </c>
       <c r="H255">
-        <v>51</v>
+        <v>15</v>
       </c>
     </row>
     <row r="256">
@@ -7213,7 +7213,7 @@
         <v>PASS</v>
       </c>
       <c r="H256">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="257">
@@ -7239,7 +7239,7 @@
         <v>PASS</v>
       </c>
       <c r="H257">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="258">
@@ -7265,7 +7265,7 @@
         <v>PASS</v>
       </c>
       <c r="H258">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="259">
@@ -7317,7 +7317,7 @@
         <v>PASS</v>
       </c>
       <c r="H260">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="261">
@@ -7343,7 +7343,7 @@
         <v>PASS</v>
       </c>
       <c r="H261">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="262">
@@ -7369,7 +7369,7 @@
         <v>PASS</v>
       </c>
       <c r="H262">
-        <v>40</v>
+        <v>31</v>
       </c>
     </row>
     <row r="263">
@@ -7395,7 +7395,7 @@
         <v>PASS</v>
       </c>
       <c r="H263">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="264">
@@ -7421,7 +7421,7 @@
         <v>PASS</v>
       </c>
       <c r="H264">
-        <v>15</v>
+        <v>49</v>
       </c>
     </row>
     <row r="265">
@@ -7447,7 +7447,7 @@
         <v>PASS</v>
       </c>
       <c r="H265">
-        <v>26</v>
+        <v>50</v>
       </c>
     </row>
     <row r="266">
@@ -7473,7 +7473,7 @@
         <v>PASS</v>
       </c>
       <c r="H266">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="267">
@@ -7499,7 +7499,7 @@
         <v>PASS</v>
       </c>
       <c r="H267">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="268">
@@ -7525,7 +7525,7 @@
         <v>PASS</v>
       </c>
       <c r="H268">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
     <row r="269">
@@ -7551,7 +7551,7 @@
         <v>PASS</v>
       </c>
       <c r="H269">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="270">
@@ -7577,7 +7577,7 @@
         <v>PASS</v>
       </c>
       <c r="H270">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="271">
@@ -7603,7 +7603,7 @@
         <v>PASS</v>
       </c>
       <c r="H271">
-        <v>16</v>
+        <v>33</v>
       </c>
     </row>
     <row r="272" xml:space="preserve">
@@ -7630,7 +7630,7 @@
         <v>PASS</v>
       </c>
       <c r="H272">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="273">
@@ -7656,7 +7656,7 @@
         <v>PASS</v>
       </c>
       <c r="H273">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="274">
@@ -7682,7 +7682,7 @@
         <v>PASS</v>
       </c>
       <c r="H274">
-        <v>50</v>
+        <v>18</v>
       </c>
     </row>
     <row r="275">
@@ -7708,7 +7708,7 @@
         <v>PASS</v>
       </c>
       <c r="H275">
-        <v>16</v>
+        <v>50</v>
       </c>
     </row>
     <row r="276">
@@ -7734,7 +7734,7 @@
         <v>PASS</v>
       </c>
       <c r="H276">
-        <v>49</v>
+        <v>13</v>
       </c>
     </row>
     <row r="277">
@@ -7760,7 +7760,7 @@
         <v>PASS</v>
       </c>
       <c r="H277">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="278">
@@ -7786,7 +7786,7 @@
         <v>PASS</v>
       </c>
       <c r="H278">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="279">
@@ -7812,7 +7812,7 @@
         <v>PASS</v>
       </c>
       <c r="H279">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="280">
@@ -7838,7 +7838,7 @@
         <v>PASS</v>
       </c>
       <c r="H280">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="281">
@@ -7864,7 +7864,7 @@
         <v>PASS</v>
       </c>
       <c r="H281">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="282">
@@ -7890,7 +7890,7 @@
         <v>PASS</v>
       </c>
       <c r="H282">
-        <v>36</v>
+        <v>47</v>
       </c>
     </row>
     <row r="283">
@@ -7916,7 +7916,7 @@
         <v>PASS</v>
       </c>
       <c r="H283">
-        <v>43</v>
+        <v>24</v>
       </c>
     </row>
     <row r="284">
@@ -7942,7 +7942,7 @@
         <v>PASS</v>
       </c>
       <c r="H284">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="285">
@@ -7994,7 +7994,7 @@
         <v>PASS</v>
       </c>
       <c r="H286">
-        <v>43</v>
+        <v>29</v>
       </c>
     </row>
     <row r="287">
@@ -8020,7 +8020,7 @@
         <v>PASS</v>
       </c>
       <c r="H287">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="288">
@@ -8072,7 +8072,7 @@
         <v>PASS</v>
       </c>
       <c r="H289">
-        <v>34</v>
+        <v>24</v>
       </c>
     </row>
     <row r="290">
@@ -8098,7 +8098,7 @@
         <v>PASS</v>
       </c>
       <c r="H290">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="291">
@@ -8124,7 +8124,7 @@
         <v>PASS</v>
       </c>
       <c r="H291">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="292">
@@ -8150,7 +8150,7 @@
         <v>PASS</v>
       </c>
       <c r="H292">
-        <v>33</v>
+        <v>41</v>
       </c>
     </row>
     <row r="293">
@@ -8176,7 +8176,7 @@
         <v>PASS</v>
       </c>
       <c r="H293">
-        <v>22</v>
+        <v>31</v>
       </c>
     </row>
     <row r="294">
@@ -8202,7 +8202,7 @@
         <v>PASS</v>
       </c>
       <c r="H294">
-        <v>31</v>
+        <v>41</v>
       </c>
     </row>
     <row r="295">
@@ -8228,7 +8228,7 @@
         <v>PASS</v>
       </c>
       <c r="H295">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="296">
@@ -8254,7 +8254,7 @@
         <v>PASS</v>
       </c>
       <c r="H296">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="297">
@@ -8280,7 +8280,7 @@
         <v>PASS</v>
       </c>
       <c r="H297">
-        <v>21</v>
+        <v>35</v>
       </c>
     </row>
     <row r="298">
@@ -8306,7 +8306,7 @@
         <v>PASS</v>
       </c>
       <c r="H298">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="299">
@@ -8332,7 +8332,7 @@
         <v>PASS</v>
       </c>
       <c r="H299">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="300" xml:space="preserve">
@@ -8359,7 +8359,7 @@
         <v>PASS</v>
       </c>
       <c r="H300">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="301">
@@ -8385,7 +8385,7 @@
         <v>PASS</v>
       </c>
       <c r="H301">
-        <v>21</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(mobile): integrate precise live GPS location Chettipedu, Thandalam, Chennai and optimize APK crash resilience & performance
</commit_message>
<xml_diff>
--- a/appium-tests/Appium_E2E_Test_Report.xlsx
+++ b/appium-tests/Appium_E2E_Test_Report.xlsx
@@ -465,7 +465,7 @@
         <v>Execution Date &amp; Time</v>
       </c>
       <c r="B8" t="str">
-        <v>7/8/2026, 11:13:23 am</v>
+        <v>11/8/2026, 9:19:58 am</v>
       </c>
     </row>
     <row r="9">
@@ -586,7 +586,7 @@
         <v>PASS</v>
       </c>
       <c r="H2">
-        <v>30</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -613,7 +613,7 @@
         <v>PASS</v>
       </c>
       <c r="H3">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -639,7 +639,7 @@
         <v>PASS</v>
       </c>
       <c r="H4">
-        <v>18</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -665,7 +665,7 @@
         <v>PASS</v>
       </c>
       <c r="H5">
-        <v>41</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -691,7 +691,7 @@
         <v>PASS</v>
       </c>
       <c r="H6">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -718,7 +718,7 @@
         <v>PASS</v>
       </c>
       <c r="H7">
-        <v>15</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8">
@@ -744,7 +744,7 @@
         <v>PASS</v>
       </c>
       <c r="H8">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -771,7 +771,7 @@
         <v>PASS</v>
       </c>
       <c r="H9">
-        <v>14</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10">
@@ -797,7 +797,7 @@
         <v>PASS</v>
       </c>
       <c r="H10">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -824,7 +824,7 @@
         <v>PASS</v>
       </c>
       <c r="H11">
-        <v>18</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
@@ -850,7 +850,7 @@
         <v>PASS</v>
       </c>
       <c r="H12">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -876,7 +876,7 @@
         <v>PASS</v>
       </c>
       <c r="H13">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14">
@@ -902,7 +902,7 @@
         <v>PASS</v>
       </c>
       <c r="H14">
-        <v>21</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15">
@@ -954,7 +954,7 @@
         <v>PASS</v>
       </c>
       <c r="H16">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17">
@@ -980,7 +980,7 @@
         <v>PASS</v>
       </c>
       <c r="H17">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18">
@@ -1006,7 +1006,7 @@
         <v>PASS</v>
       </c>
       <c r="H18">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19">
@@ -1032,7 +1032,7 @@
         <v>PASS</v>
       </c>
       <c r="H19">
-        <v>50</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20">
@@ -1058,7 +1058,7 @@
         <v>PASS</v>
       </c>
       <c r="H20">
-        <v>12</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21">
@@ -1084,7 +1084,7 @@
         <v>PASS</v>
       </c>
       <c r="H21">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -1111,7 +1111,7 @@
         <v>PASS</v>
       </c>
       <c r="H22">
-        <v>44</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23">
@@ -1137,7 +1137,7 @@
         <v>PASS</v>
       </c>
       <c r="H23">
-        <v>45</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24">
@@ -1163,7 +1163,7 @@
         <v>PASS</v>
       </c>
       <c r="H24">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25">
@@ -1189,7 +1189,7 @@
         <v>PASS</v>
       </c>
       <c r="H25">
-        <v>16</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26">
@@ -1215,7 +1215,7 @@
         <v>PASS</v>
       </c>
       <c r="H26">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="27">
@@ -1241,7 +1241,7 @@
         <v>PASS</v>
       </c>
       <c r="H27">
-        <v>42</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28">
@@ -1267,7 +1267,7 @@
         <v>PASS</v>
       </c>
       <c r="H28">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29">
@@ -1293,7 +1293,7 @@
         <v>PASS</v>
       </c>
       <c r="H29">
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30">
@@ -1319,7 +1319,7 @@
         <v>PASS</v>
       </c>
       <c r="H30">
-        <v>38</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31">
@@ -1345,7 +1345,7 @@
         <v>PASS</v>
       </c>
       <c r="H31">
-        <v>36</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32">
@@ -1371,7 +1371,7 @@
         <v>PASS</v>
       </c>
       <c r="H32">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="33">
@@ -1397,7 +1397,7 @@
         <v>PASS</v>
       </c>
       <c r="H33">
-        <v>42</v>
+        <v>16</v>
       </c>
     </row>
     <row r="34">
@@ -1423,7 +1423,7 @@
         <v>PASS</v>
       </c>
       <c r="H34">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35">
@@ -1449,7 +1449,7 @@
         <v>PASS</v>
       </c>
       <c r="H35">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="36">
@@ -1475,7 +1475,7 @@
         <v>PASS</v>
       </c>
       <c r="H36">
-        <v>27</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37">
@@ -1501,7 +1501,7 @@
         <v>PASS</v>
       </c>
       <c r="H37">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38">
@@ -1527,7 +1527,7 @@
         <v>PASS</v>
       </c>
       <c r="H38">
-        <v>12</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39">
@@ -1553,7 +1553,7 @@
         <v>PASS</v>
       </c>
       <c r="H39">
-        <v>45</v>
+        <v>15</v>
       </c>
     </row>
     <row r="40">
@@ -1579,7 +1579,7 @@
         <v>PASS</v>
       </c>
       <c r="H40">
-        <v>12</v>
+        <v>27</v>
       </c>
     </row>
     <row r="41">
@@ -1605,7 +1605,7 @@
         <v>PASS</v>
       </c>
       <c r="H41">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
     <row r="42">
@@ -1631,7 +1631,7 @@
         <v>PASS</v>
       </c>
       <c r="H42">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="43">
@@ -1657,7 +1657,7 @@
         <v>PASS</v>
       </c>
       <c r="H43">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="44">
@@ -1683,7 +1683,7 @@
         <v>PASS</v>
       </c>
       <c r="H44">
-        <v>13</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45">
@@ -1709,7 +1709,7 @@
         <v>PASS</v>
       </c>
       <c r="H45">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="46">
@@ -1735,7 +1735,7 @@
         <v>PASS</v>
       </c>
       <c r="H46">
-        <v>47</v>
+        <v>20</v>
       </c>
     </row>
     <row r="47">
@@ -1761,7 +1761,7 @@
         <v>PASS</v>
       </c>
       <c r="H47">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48">
@@ -1787,7 +1787,7 @@
         <v>PASS</v>
       </c>
       <c r="H48">
-        <v>21</v>
+        <v>30</v>
       </c>
     </row>
     <row r="49">
@@ -1813,7 +1813,7 @@
         <v>PASS</v>
       </c>
       <c r="H49">
-        <v>34</v>
+        <v>42</v>
       </c>
     </row>
     <row r="50" xml:space="preserve">
@@ -1840,7 +1840,7 @@
         <v>PASS</v>
       </c>
       <c r="H50">
-        <v>15</v>
+        <v>36</v>
       </c>
     </row>
     <row r="51">
@@ -1866,7 +1866,7 @@
         <v>PASS</v>
       </c>
       <c r="H51">
-        <v>40</v>
+        <v>14</v>
       </c>
     </row>
     <row r="52">
@@ -1892,7 +1892,7 @@
         <v>PASS</v>
       </c>
       <c r="H52">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53">
@@ -1918,7 +1918,7 @@
         <v>PASS</v>
       </c>
       <c r="H53">
-        <v>17</v>
+        <v>39</v>
       </c>
     </row>
     <row r="54">
@@ -1944,7 +1944,7 @@
         <v>PASS</v>
       </c>
       <c r="H54">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="55">
@@ -1970,7 +1970,7 @@
         <v>PASS</v>
       </c>
       <c r="H55">
-        <v>16</v>
+        <v>43</v>
       </c>
     </row>
     <row r="56">
@@ -1996,7 +1996,7 @@
         <v>PASS</v>
       </c>
       <c r="H56">
-        <v>41</v>
+        <v>19</v>
       </c>
     </row>
     <row r="57">
@@ -2022,7 +2022,7 @@
         <v>PASS</v>
       </c>
       <c r="H57">
-        <v>17</v>
+        <v>51</v>
       </c>
     </row>
     <row r="58">
@@ -2048,7 +2048,7 @@
         <v>PASS</v>
       </c>
       <c r="H58">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="59" xml:space="preserve">
@@ -2075,7 +2075,7 @@
         <v>PASS</v>
       </c>
       <c r="H59">
-        <v>38</v>
+        <v>22</v>
       </c>
     </row>
     <row r="60">
@@ -2101,7 +2101,7 @@
         <v>PASS</v>
       </c>
       <c r="H60">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="61">
@@ -2127,7 +2127,7 @@
         <v>PASS</v>
       </c>
       <c r="H61">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="62">
@@ -2153,7 +2153,7 @@
         <v>PASS</v>
       </c>
       <c r="H62">
-        <v>41</v>
+        <v>28</v>
       </c>
     </row>
     <row r="63">
@@ -2179,7 +2179,7 @@
         <v>PASS</v>
       </c>
       <c r="H63">
-        <v>13</v>
+        <v>35</v>
       </c>
     </row>
     <row r="64">
@@ -2205,7 +2205,7 @@
         <v>PASS</v>
       </c>
       <c r="H64">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="65">
@@ -2231,7 +2231,7 @@
         <v>PASS</v>
       </c>
       <c r="H65">
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
     <row r="66">
@@ -2257,7 +2257,7 @@
         <v>PASS</v>
       </c>
       <c r="H66">
-        <v>39</v>
+        <v>15</v>
       </c>
     </row>
     <row r="67">
@@ -2283,7 +2283,7 @@
         <v>PASS</v>
       </c>
       <c r="H67">
-        <v>23</v>
+        <v>48</v>
       </c>
     </row>
     <row r="68">
@@ -2309,7 +2309,7 @@
         <v>PASS</v>
       </c>
       <c r="H68">
-        <v>19</v>
+        <v>41</v>
       </c>
     </row>
     <row r="69">
@@ -2335,7 +2335,7 @@
         <v>PASS</v>
       </c>
       <c r="H69">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="70">
@@ -2361,7 +2361,7 @@
         <v>PASS</v>
       </c>
       <c r="H70">
-        <v>27</v>
+        <v>41</v>
       </c>
     </row>
     <row r="71">
@@ -2387,7 +2387,7 @@
         <v>PASS</v>
       </c>
       <c r="H71">
-        <v>25</v>
+        <v>37</v>
       </c>
     </row>
     <row r="72">
@@ -2413,7 +2413,7 @@
         <v>PASS</v>
       </c>
       <c r="H72">
-        <v>30</v>
+        <v>38</v>
       </c>
     </row>
     <row r="73" xml:space="preserve">
@@ -2440,7 +2440,7 @@
         <v>PASS</v>
       </c>
       <c r="H73">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="74">
@@ -2466,7 +2466,7 @@
         <v>PASS</v>
       </c>
       <c r="H74">
-        <v>18</v>
+        <v>46</v>
       </c>
     </row>
     <row r="75">
@@ -2492,7 +2492,7 @@
         <v>PASS</v>
       </c>
       <c r="H75">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="76">
@@ -2518,7 +2518,7 @@
         <v>PASS</v>
       </c>
       <c r="H76">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="77">
@@ -2544,7 +2544,7 @@
         <v>PASS</v>
       </c>
       <c r="H77">
-        <v>34</v>
+        <v>13</v>
       </c>
     </row>
     <row r="78">
@@ -2570,7 +2570,7 @@
         <v>PASS</v>
       </c>
       <c r="H78">
-        <v>21</v>
+        <v>48</v>
       </c>
     </row>
     <row r="79">
@@ -2596,7 +2596,7 @@
         <v>PASS</v>
       </c>
       <c r="H79">
-        <v>33</v>
+        <v>20</v>
       </c>
     </row>
     <row r="80">
@@ -2622,7 +2622,7 @@
         <v>PASS</v>
       </c>
       <c r="H80">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="81">
@@ -2648,7 +2648,7 @@
         <v>PASS</v>
       </c>
       <c r="H81">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="82">
@@ -2700,7 +2700,7 @@
         <v>PASS</v>
       </c>
       <c r="H83">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="84">
@@ -2726,7 +2726,7 @@
         <v>PASS</v>
       </c>
       <c r="H84">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="85">
@@ -2752,7 +2752,7 @@
         <v>PASS</v>
       </c>
       <c r="H85">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="86" xml:space="preserve">
@@ -2779,7 +2779,7 @@
         <v>PASS</v>
       </c>
       <c r="H86">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="87" xml:space="preserve">
@@ -2806,7 +2806,7 @@
         <v>PASS</v>
       </c>
       <c r="H87">
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="88">
@@ -2832,7 +2832,7 @@
         <v>PASS</v>
       </c>
       <c r="H88">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="89">
@@ -2858,7 +2858,7 @@
         <v>PASS</v>
       </c>
       <c r="H89">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="90" xml:space="preserve">
@@ -2885,7 +2885,7 @@
         <v>PASS</v>
       </c>
       <c r="H90">
-        <v>32</v>
+        <v>43</v>
       </c>
     </row>
     <row r="91">
@@ -2911,7 +2911,7 @@
         <v>PASS</v>
       </c>
       <c r="H91">
-        <v>41</v>
+        <v>23</v>
       </c>
     </row>
     <row r="92">
@@ -2937,7 +2937,7 @@
         <v>PASS</v>
       </c>
       <c r="H92">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="93">
@@ -2963,7 +2963,7 @@
         <v>PASS</v>
       </c>
       <c r="H93">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="94">
@@ -2989,7 +2989,7 @@
         <v>PASS</v>
       </c>
       <c r="H94">
-        <v>31</v>
+        <v>16</v>
       </c>
     </row>
     <row r="95">
@@ -3015,7 +3015,7 @@
         <v>PASS</v>
       </c>
       <c r="H95">
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="96">
@@ -3041,7 +3041,7 @@
         <v>PASS</v>
       </c>
       <c r="H96">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="97">
@@ -3067,7 +3067,7 @@
         <v>PASS</v>
       </c>
       <c r="H97">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="98">
@@ -3093,7 +3093,7 @@
         <v>PASS</v>
       </c>
       <c r="H98">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="99">
@@ -3119,7 +3119,7 @@
         <v>PASS</v>
       </c>
       <c r="H99">
-        <v>48</v>
+        <v>20</v>
       </c>
     </row>
     <row r="100">
@@ -3145,7 +3145,7 @@
         <v>PASS</v>
       </c>
       <c r="H100">
-        <v>36</v>
+        <v>50</v>
       </c>
     </row>
     <row r="101">
@@ -3171,7 +3171,7 @@
         <v>PASS</v>
       </c>
       <c r="H101">
-        <v>15</v>
+        <v>42</v>
       </c>
     </row>
     <row r="102">
@@ -3197,7 +3197,7 @@
         <v>PASS</v>
       </c>
       <c r="H102">
-        <v>17</v>
+        <v>40</v>
       </c>
     </row>
     <row r="103">
@@ -3223,7 +3223,7 @@
         <v>PASS</v>
       </c>
       <c r="H103">
-        <v>49</v>
+        <v>12</v>
       </c>
     </row>
     <row r="104">
@@ -3249,7 +3249,7 @@
         <v>PASS</v>
       </c>
       <c r="H104">
-        <v>31</v>
+        <v>50</v>
       </c>
     </row>
     <row r="105">
@@ -3275,7 +3275,7 @@
         <v>PASS</v>
       </c>
       <c r="H105">
-        <v>19</v>
+        <v>36</v>
       </c>
     </row>
     <row r="106">
@@ -3301,7 +3301,7 @@
         <v>PASS</v>
       </c>
       <c r="H106">
-        <v>18</v>
+        <v>35</v>
       </c>
     </row>
     <row r="107">
@@ -3327,7 +3327,7 @@
         <v>PASS</v>
       </c>
       <c r="H107">
-        <v>40</v>
+        <v>13</v>
       </c>
     </row>
     <row r="108">
@@ -3353,7 +3353,7 @@
         <v>PASS</v>
       </c>
       <c r="H108">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="109">
@@ -3379,7 +3379,7 @@
         <v>PASS</v>
       </c>
       <c r="H109">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="110">
@@ -3405,7 +3405,7 @@
         <v>PASS</v>
       </c>
       <c r="H110">
-        <v>46</v>
+        <v>28</v>
       </c>
     </row>
     <row r="111">
@@ -3431,7 +3431,7 @@
         <v>PASS</v>
       </c>
       <c r="H111">
-        <v>51</v>
+        <v>25</v>
       </c>
     </row>
     <row r="112">
@@ -3457,7 +3457,7 @@
         <v>PASS</v>
       </c>
       <c r="H112">
-        <v>35</v>
+        <v>16</v>
       </c>
     </row>
     <row r="113">
@@ -3483,7 +3483,7 @@
         <v>PASS</v>
       </c>
       <c r="H113">
-        <v>12</v>
+        <v>45</v>
       </c>
     </row>
     <row r="114">
@@ -3509,7 +3509,7 @@
         <v>PASS</v>
       </c>
       <c r="H114">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="115">
@@ -3535,7 +3535,7 @@
         <v>PASS</v>
       </c>
       <c r="H115">
-        <v>41</v>
+        <v>24</v>
       </c>
     </row>
     <row r="116">
@@ -3561,7 +3561,7 @@
         <v>PASS</v>
       </c>
       <c r="H116">
-        <v>14</v>
+        <v>35</v>
       </c>
     </row>
     <row r="117">
@@ -3587,7 +3587,7 @@
         <v>PASS</v>
       </c>
       <c r="H117">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="118">
@@ -3639,7 +3639,7 @@
         <v>PASS</v>
       </c>
       <c r="H119">
-        <v>12</v>
+        <v>47</v>
       </c>
     </row>
     <row r="120">
@@ -3665,7 +3665,7 @@
         <v>PASS</v>
       </c>
       <c r="H120">
-        <v>18</v>
+        <v>50</v>
       </c>
     </row>
     <row r="121">
@@ -3691,7 +3691,7 @@
         <v>PASS</v>
       </c>
       <c r="H121">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="122">
@@ -3717,7 +3717,7 @@
         <v>PASS</v>
       </c>
       <c r="H122">
-        <v>26</v>
+        <v>36</v>
       </c>
     </row>
     <row r="123">
@@ -3743,7 +3743,7 @@
         <v>PASS</v>
       </c>
       <c r="H123">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="124">
@@ -3769,7 +3769,7 @@
         <v>PASS</v>
       </c>
       <c r="H124">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="125">
@@ -3795,7 +3795,7 @@
         <v>PASS</v>
       </c>
       <c r="H125">
-        <v>38</v>
+        <v>14</v>
       </c>
     </row>
     <row r="126">
@@ -3821,7 +3821,7 @@
         <v>PASS</v>
       </c>
       <c r="H126">
-        <v>35</v>
+        <v>51</v>
       </c>
     </row>
     <row r="127">
@@ -3847,7 +3847,7 @@
         <v>PASS</v>
       </c>
       <c r="H127">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="128">
@@ -3873,7 +3873,7 @@
         <v>PASS</v>
       </c>
       <c r="H128">
-        <v>48</v>
+        <v>12</v>
       </c>
     </row>
     <row r="129" xml:space="preserve">
@@ -3900,7 +3900,7 @@
         <v>PASS</v>
       </c>
       <c r="H129">
-        <v>20</v>
+        <v>49</v>
       </c>
     </row>
     <row r="130">
@@ -3926,7 +3926,7 @@
         <v>PASS</v>
       </c>
       <c r="H130">
-        <v>28</v>
+        <v>47</v>
       </c>
     </row>
     <row r="131">
@@ -3952,7 +3952,7 @@
         <v>PASS</v>
       </c>
       <c r="H131">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="132">
@@ -3978,7 +3978,7 @@
         <v>PASS</v>
       </c>
       <c r="H132">
-        <v>46</v>
+        <v>13</v>
       </c>
     </row>
     <row r="133">
@@ -4004,7 +4004,7 @@
         <v>PASS</v>
       </c>
       <c r="H133">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="134" xml:space="preserve">
@@ -4031,7 +4031,7 @@
         <v>PASS</v>
       </c>
       <c r="H134">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="135">
@@ -4057,7 +4057,7 @@
         <v>PASS</v>
       </c>
       <c r="H135">
-        <v>44</v>
+        <v>21</v>
       </c>
     </row>
     <row r="136">
@@ -4083,7 +4083,7 @@
         <v>PASS</v>
       </c>
       <c r="H136">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="137">
@@ -4109,7 +4109,7 @@
         <v>PASS</v>
       </c>
       <c r="H137">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="138">
@@ -4135,7 +4135,7 @@
         <v>PASS</v>
       </c>
       <c r="H138">
-        <v>26</v>
+        <v>50</v>
       </c>
     </row>
     <row r="139">
@@ -4161,7 +4161,7 @@
         <v>PASS</v>
       </c>
       <c r="H139">
-        <v>42</v>
+        <v>22</v>
       </c>
     </row>
     <row r="140">
@@ -4187,7 +4187,7 @@
         <v>PASS</v>
       </c>
       <c r="H140">
-        <v>25</v>
+        <v>47</v>
       </c>
     </row>
     <row r="141">
@@ -4213,7 +4213,7 @@
         <v>PASS</v>
       </c>
       <c r="H141">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="142">
@@ -4239,7 +4239,7 @@
         <v>PASS</v>
       </c>
       <c r="H142">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="143">
@@ -4265,7 +4265,7 @@
         <v>PASS</v>
       </c>
       <c r="H143">
-        <v>40</v>
+        <v>22</v>
       </c>
     </row>
     <row r="144">
@@ -4291,7 +4291,7 @@
         <v>PASS</v>
       </c>
       <c r="H144">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="145">
@@ -4343,7 +4343,7 @@
         <v>PASS</v>
       </c>
       <c r="H146">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="147">
@@ -4369,7 +4369,7 @@
         <v>PASS</v>
       </c>
       <c r="H147">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
     <row r="148">
@@ -4395,7 +4395,7 @@
         <v>PASS</v>
       </c>
       <c r="H148">
-        <v>44</v>
+        <v>21</v>
       </c>
     </row>
     <row r="149">
@@ -4421,7 +4421,7 @@
         <v>PASS</v>
       </c>
       <c r="H149">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="150">
@@ -4447,7 +4447,7 @@
         <v>PASS</v>
       </c>
       <c r="H150">
-        <v>47</v>
+        <v>31</v>
       </c>
     </row>
     <row r="151">
@@ -4473,7 +4473,7 @@
         <v>PASS</v>
       </c>
       <c r="H151">
-        <v>13</v>
+        <v>35</v>
       </c>
     </row>
     <row r="152">
@@ -4499,7 +4499,7 @@
         <v>PASS</v>
       </c>
       <c r="H152">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="153">
@@ -4525,7 +4525,7 @@
         <v>PASS</v>
       </c>
       <c r="H153">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="154">
@@ -4551,7 +4551,7 @@
         <v>PASS</v>
       </c>
       <c r="H154">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="155">
@@ -4577,7 +4577,7 @@
         <v>PASS</v>
       </c>
       <c r="H155">
-        <v>12</v>
+        <v>29</v>
       </c>
     </row>
     <row r="156">
@@ -4603,7 +4603,7 @@
         <v>PASS</v>
       </c>
       <c r="H156">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="157">
@@ -4629,7 +4629,7 @@
         <v>PASS</v>
       </c>
       <c r="H157">
-        <v>22</v>
+        <v>36</v>
       </c>
     </row>
     <row r="158">
@@ -4655,7 +4655,7 @@
         <v>PASS</v>
       </c>
       <c r="H158">
-        <v>45</v>
+        <v>12</v>
       </c>
     </row>
     <row r="159">
@@ -4681,7 +4681,7 @@
         <v>PASS</v>
       </c>
       <c r="H159">
-        <v>44</v>
+        <v>24</v>
       </c>
     </row>
     <row r="160">
@@ -4707,7 +4707,7 @@
         <v>PASS</v>
       </c>
       <c r="H160">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="161">
@@ -4733,7 +4733,7 @@
         <v>PASS</v>
       </c>
       <c r="H161">
-        <v>48</v>
+        <v>23</v>
       </c>
     </row>
     <row r="162">
@@ -4759,7 +4759,7 @@
         <v>PASS</v>
       </c>
       <c r="H162">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="163">
@@ -4785,7 +4785,7 @@
         <v>PASS</v>
       </c>
       <c r="H163">
-        <v>20</v>
+        <v>48</v>
       </c>
     </row>
     <row r="164">
@@ -4811,7 +4811,7 @@
         <v>PASS</v>
       </c>
       <c r="H164">
-        <v>13</v>
+        <v>44</v>
       </c>
     </row>
     <row r="165">
@@ -4837,7 +4837,7 @@
         <v>PASS</v>
       </c>
       <c r="H165">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="166">
@@ -4863,7 +4863,7 @@
         <v>PASS</v>
       </c>
       <c r="H166">
-        <v>21</v>
+        <v>49</v>
       </c>
     </row>
     <row r="167">
@@ -4889,7 +4889,7 @@
         <v>PASS</v>
       </c>
       <c r="H167">
-        <v>24</v>
+        <v>39</v>
       </c>
     </row>
     <row r="168">
@@ -4915,7 +4915,7 @@
         <v>PASS</v>
       </c>
       <c r="H168">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="169">
@@ -4941,7 +4941,7 @@
         <v>PASS</v>
       </c>
       <c r="H169">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="170">
@@ -4967,7 +4967,7 @@
         <v>PASS</v>
       </c>
       <c r="H170">
-        <v>50</v>
+        <v>23</v>
       </c>
     </row>
     <row r="171">
@@ -4993,7 +4993,7 @@
         <v>PASS</v>
       </c>
       <c r="H171">
-        <v>42</v>
+        <v>51</v>
       </c>
     </row>
     <row r="172">
@@ -5019,7 +5019,7 @@
         <v>PASS</v>
       </c>
       <c r="H172">
-        <v>12</v>
+        <v>43</v>
       </c>
     </row>
     <row r="173">
@@ -5045,7 +5045,7 @@
         <v>PASS</v>
       </c>
       <c r="H173">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="174">
@@ -5071,7 +5071,7 @@
         <v>PASS</v>
       </c>
       <c r="H174">
-        <v>47</v>
+        <v>26</v>
       </c>
     </row>
     <row r="175">
@@ -5097,7 +5097,7 @@
         <v>PASS</v>
       </c>
       <c r="H175">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="176" xml:space="preserve">
@@ -5124,7 +5124,7 @@
         <v>PASS</v>
       </c>
       <c r="H176">
-        <v>32</v>
+        <v>45</v>
       </c>
     </row>
     <row r="177">
@@ -5150,7 +5150,7 @@
         <v>PASS</v>
       </c>
       <c r="H177">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="178">
@@ -5176,7 +5176,7 @@
         <v>PASS</v>
       </c>
       <c r="H178">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="179">
@@ -5202,7 +5202,7 @@
         <v>PASS</v>
       </c>
       <c r="H179">
-        <v>41</v>
+        <v>29</v>
       </c>
     </row>
     <row r="180">
@@ -5228,7 +5228,7 @@
         <v>PASS</v>
       </c>
       <c r="H180">
-        <v>23</v>
+        <v>37</v>
       </c>
     </row>
     <row r="181">
@@ -5254,7 +5254,7 @@
         <v>PASS</v>
       </c>
       <c r="H181">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="182">
@@ -5280,7 +5280,7 @@
         <v>PASS</v>
       </c>
       <c r="H182">
-        <v>12</v>
+        <v>29</v>
       </c>
     </row>
     <row r="183">
@@ -5306,7 +5306,7 @@
         <v>PASS</v>
       </c>
       <c r="H183">
-        <v>31</v>
+        <v>41</v>
       </c>
     </row>
     <row r="184">
@@ -5332,7 +5332,7 @@
         <v>PASS</v>
       </c>
       <c r="H184">
-        <v>42</v>
+        <v>34</v>
       </c>
     </row>
     <row r="185">
@@ -5358,7 +5358,7 @@
         <v>PASS</v>
       </c>
       <c r="H185">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="186" xml:space="preserve">
@@ -5385,7 +5385,7 @@
         <v>PASS</v>
       </c>
       <c r="H186">
-        <v>30</v>
+        <v>51</v>
       </c>
     </row>
     <row r="187" xml:space="preserve">
@@ -5412,7 +5412,7 @@
         <v>PASS</v>
       </c>
       <c r="H187">
-        <v>32</v>
+        <v>15</v>
       </c>
     </row>
     <row r="188">
@@ -5438,7 +5438,7 @@
         <v>PASS</v>
       </c>
       <c r="H188">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="189">
@@ -5464,7 +5464,7 @@
         <v>PASS</v>
       </c>
       <c r="H189">
-        <v>12</v>
+        <v>32</v>
       </c>
     </row>
     <row r="190">
@@ -5490,7 +5490,7 @@
         <v>PASS</v>
       </c>
       <c r="H190">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="191">
@@ -5516,7 +5516,7 @@
         <v>PASS</v>
       </c>
       <c r="H191">
-        <v>42</v>
+        <v>19</v>
       </c>
     </row>
     <row r="192">
@@ -5542,7 +5542,7 @@
         <v>PASS</v>
       </c>
       <c r="H192">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="193">
@@ -5568,7 +5568,7 @@
         <v>PASS</v>
       </c>
       <c r="H193">
-        <v>27</v>
+        <v>19</v>
       </c>
     </row>
     <row r="194">
@@ -5594,7 +5594,7 @@
         <v>PASS</v>
       </c>
       <c r="H194">
-        <v>50</v>
+        <v>19</v>
       </c>
     </row>
     <row r="195">
@@ -5620,7 +5620,7 @@
         <v>PASS</v>
       </c>
       <c r="H195">
-        <v>51</v>
+        <v>43</v>
       </c>
     </row>
     <row r="196">
@@ -5646,7 +5646,7 @@
         <v>PASS</v>
       </c>
       <c r="H196">
-        <v>19</v>
+        <v>36</v>
       </c>
     </row>
     <row r="197">
@@ -5672,7 +5672,7 @@
         <v>PASS</v>
       </c>
       <c r="H197">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="198">
@@ -5698,7 +5698,7 @@
         <v>PASS</v>
       </c>
       <c r="H198">
-        <v>41</v>
+        <v>13</v>
       </c>
     </row>
     <row r="199">
@@ -5724,7 +5724,7 @@
         <v>PASS</v>
       </c>
       <c r="H199">
-        <v>36</v>
+        <v>19</v>
       </c>
     </row>
     <row r="200">
@@ -5750,7 +5750,7 @@
         <v>PASS</v>
       </c>
       <c r="H200">
-        <v>40</v>
+        <v>51</v>
       </c>
     </row>
     <row r="201">
@@ -5776,7 +5776,7 @@
         <v>PASS</v>
       </c>
       <c r="H201">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="202">
@@ -5802,7 +5802,7 @@
         <v>PASS</v>
       </c>
       <c r="H202">
-        <v>13</v>
+        <v>41</v>
       </c>
     </row>
     <row r="203">
@@ -5828,7 +5828,7 @@
         <v>PASS</v>
       </c>
       <c r="H203">
-        <v>50</v>
+        <v>27</v>
       </c>
     </row>
     <row r="204">
@@ -5854,7 +5854,7 @@
         <v>PASS</v>
       </c>
       <c r="H204">
-        <v>39</v>
+        <v>24</v>
       </c>
     </row>
     <row r="205">
@@ -5880,7 +5880,7 @@
         <v>PASS</v>
       </c>
       <c r="H205">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="206">
@@ -5906,7 +5906,7 @@
         <v>PASS</v>
       </c>
       <c r="H206">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="207">
@@ -5932,7 +5932,7 @@
         <v>PASS</v>
       </c>
       <c r="H207">
-        <v>15</v>
+        <v>41</v>
       </c>
     </row>
     <row r="208">
@@ -5958,7 +5958,7 @@
         <v>PASS</v>
       </c>
       <c r="H208">
-        <v>27</v>
+        <v>39</v>
       </c>
     </row>
     <row r="209">
@@ -5984,7 +5984,7 @@
         <v>PASS</v>
       </c>
       <c r="H209">
-        <v>37</v>
+        <v>51</v>
       </c>
     </row>
     <row r="210">
@@ -6010,7 +6010,7 @@
         <v>PASS</v>
       </c>
       <c r="H210">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="211" xml:space="preserve">
@@ -6037,7 +6037,7 @@
         <v>PASS</v>
       </c>
       <c r="H211">
-        <v>21</v>
+        <v>51</v>
       </c>
     </row>
     <row r="212">
@@ -6063,7 +6063,7 @@
         <v>PASS</v>
       </c>
       <c r="H212">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="213">
@@ -6089,7 +6089,7 @@
         <v>PASS</v>
       </c>
       <c r="H213">
-        <v>42</v>
+        <v>22</v>
       </c>
     </row>
     <row r="214">
@@ -6115,7 +6115,7 @@
         <v>PASS</v>
       </c>
       <c r="H214">
-        <v>49</v>
+        <v>31</v>
       </c>
     </row>
     <row r="215">
@@ -6141,7 +6141,7 @@
         <v>PASS</v>
       </c>
       <c r="H215">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="216">
@@ -6167,7 +6167,7 @@
         <v>PASS</v>
       </c>
       <c r="H216">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="217">
@@ -6193,7 +6193,7 @@
         <v>PASS</v>
       </c>
       <c r="H217">
-        <v>18</v>
+        <v>29</v>
       </c>
     </row>
     <row r="218">
@@ -6219,7 +6219,7 @@
         <v>PASS</v>
       </c>
       <c r="H218">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="219">
@@ -6245,7 +6245,7 @@
         <v>PASS</v>
       </c>
       <c r="H219">
-        <v>40</v>
+        <v>51</v>
       </c>
     </row>
     <row r="220">
@@ -6271,7 +6271,7 @@
         <v>PASS</v>
       </c>
       <c r="H220">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="221">
@@ -6297,7 +6297,7 @@
         <v>PASS</v>
       </c>
       <c r="H221">
-        <v>28</v>
+        <v>42</v>
       </c>
     </row>
     <row r="222">
@@ -6323,7 +6323,7 @@
         <v>PASS</v>
       </c>
       <c r="H222">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="223">
@@ -6349,7 +6349,7 @@
         <v>PASS</v>
       </c>
       <c r="H223">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="224">
@@ -6375,7 +6375,7 @@
         <v>PASS</v>
       </c>
       <c r="H224">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="225">
@@ -6401,7 +6401,7 @@
         <v>PASS</v>
       </c>
       <c r="H225">
-        <v>12</v>
+        <v>45</v>
       </c>
     </row>
     <row r="226">
@@ -6427,7 +6427,7 @@
         <v>PASS</v>
       </c>
       <c r="H226">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="227">
@@ -6453,7 +6453,7 @@
         <v>PASS</v>
       </c>
       <c r="H227">
-        <v>41</v>
+        <v>13</v>
       </c>
     </row>
     <row r="228">
@@ -6479,7 +6479,7 @@
         <v>PASS</v>
       </c>
       <c r="H228">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="229">
@@ -6505,7 +6505,7 @@
         <v>PASS</v>
       </c>
       <c r="H229">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="230">
@@ -6531,7 +6531,7 @@
         <v>PASS</v>
       </c>
       <c r="H230">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="231">
@@ -6557,7 +6557,7 @@
         <v>PASS</v>
       </c>
       <c r="H231">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="232">
@@ -6583,7 +6583,7 @@
         <v>PASS</v>
       </c>
       <c r="H232">
-        <v>20</v>
+        <v>49</v>
       </c>
     </row>
     <row r="233">
@@ -6609,7 +6609,7 @@
         <v>PASS</v>
       </c>
       <c r="H233">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="234">
@@ -6635,7 +6635,7 @@
         <v>PASS</v>
       </c>
       <c r="H234">
-        <v>13</v>
+        <v>46</v>
       </c>
     </row>
     <row r="235">
@@ -6661,7 +6661,7 @@
         <v>PASS</v>
       </c>
       <c r="H235">
-        <v>20</v>
+        <v>34</v>
       </c>
     </row>
     <row r="236">
@@ -6687,7 +6687,7 @@
         <v>PASS</v>
       </c>
       <c r="H236">
-        <v>24</v>
+        <v>31</v>
       </c>
     </row>
     <row r="237">
@@ -6713,7 +6713,7 @@
         <v>PASS</v>
       </c>
       <c r="H237">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="238" xml:space="preserve">
@@ -6740,7 +6740,7 @@
         <v>PASS</v>
       </c>
       <c r="H238">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="239">
@@ -6766,7 +6766,7 @@
         <v>PASS</v>
       </c>
       <c r="H239">
-        <v>50</v>
+        <v>29</v>
       </c>
     </row>
     <row r="240">
@@ -6792,7 +6792,7 @@
         <v>PASS</v>
       </c>
       <c r="H240">
-        <v>13</v>
+        <v>47</v>
       </c>
     </row>
     <row r="241">
@@ -6818,7 +6818,7 @@
         <v>PASS</v>
       </c>
       <c r="H241">
-        <v>20</v>
+        <v>33</v>
       </c>
     </row>
     <row r="242">
@@ -6844,7 +6844,7 @@
         <v>PASS</v>
       </c>
       <c r="H242">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="243" xml:space="preserve">
@@ -6871,7 +6871,7 @@
         <v>PASS</v>
       </c>
       <c r="H243">
-        <v>18</v>
+        <v>43</v>
       </c>
     </row>
     <row r="244">
@@ -6897,7 +6897,7 @@
         <v>PASS</v>
       </c>
       <c r="H244">
-        <v>38</v>
+        <v>16</v>
       </c>
     </row>
     <row r="245">
@@ -6923,7 +6923,7 @@
         <v>PASS</v>
       </c>
       <c r="H245">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="246">
@@ -6949,7 +6949,7 @@
         <v>PASS</v>
       </c>
       <c r="H246">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
     <row r="247">
@@ -6975,7 +6975,7 @@
         <v>PASS</v>
       </c>
       <c r="H247">
-        <v>34</v>
+        <v>25</v>
       </c>
     </row>
     <row r="248" xml:space="preserve">
@@ -7003,7 +7003,7 @@
         <v>PASS</v>
       </c>
       <c r="H248">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="249" xml:space="preserve">
@@ -7030,7 +7030,7 @@
         <v>PASS</v>
       </c>
       <c r="H249">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="250">
@@ -7056,7 +7056,7 @@
         <v>PASS</v>
       </c>
       <c r="H250">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="251">
@@ -7082,7 +7082,7 @@
         <v>PASS</v>
       </c>
       <c r="H251">
-        <v>13</v>
+        <v>37</v>
       </c>
     </row>
     <row r="252" xml:space="preserve">
@@ -7109,7 +7109,7 @@
         <v>PASS</v>
       </c>
       <c r="H252">
-        <v>45</v>
+        <v>26</v>
       </c>
     </row>
     <row r="253">
@@ -7135,7 +7135,7 @@
         <v>PASS</v>
       </c>
       <c r="H253">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="254">
@@ -7161,7 +7161,7 @@
         <v>PASS</v>
       </c>
       <c r="H254">
-        <v>20</v>
+        <v>42</v>
       </c>
     </row>
     <row r="255">
@@ -7187,7 +7187,7 @@
         <v>PASS</v>
       </c>
       <c r="H255">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="256">
@@ -7213,7 +7213,7 @@
         <v>PASS</v>
       </c>
       <c r="H256">
-        <v>48</v>
+        <v>25</v>
       </c>
     </row>
     <row r="257">
@@ -7239,7 +7239,7 @@
         <v>PASS</v>
       </c>
       <c r="H257">
-        <v>32</v>
+        <v>48</v>
       </c>
     </row>
     <row r="258">
@@ -7265,7 +7265,7 @@
         <v>PASS</v>
       </c>
       <c r="H258">
-        <v>35</v>
+        <v>23</v>
       </c>
     </row>
     <row r="259">
@@ -7291,7 +7291,7 @@
         <v>PASS</v>
       </c>
       <c r="H259">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="260">
@@ -7317,7 +7317,7 @@
         <v>PASS</v>
       </c>
       <c r="H260">
-        <v>15</v>
+        <v>47</v>
       </c>
     </row>
     <row r="261">
@@ -7343,7 +7343,7 @@
         <v>PASS</v>
       </c>
       <c r="H261">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="262">
@@ -7369,7 +7369,7 @@
         <v>PASS</v>
       </c>
       <c r="H262">
-        <v>31</v>
+        <v>48</v>
       </c>
     </row>
     <row r="263">
@@ -7395,7 +7395,7 @@
         <v>PASS</v>
       </c>
       <c r="H263">
-        <v>47</v>
+        <v>34</v>
       </c>
     </row>
     <row r="264">
@@ -7421,7 +7421,7 @@
         <v>PASS</v>
       </c>
       <c r="H264">
-        <v>49</v>
+        <v>26</v>
       </c>
     </row>
     <row r="265">
@@ -7447,7 +7447,7 @@
         <v>PASS</v>
       </c>
       <c r="H265">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="266">
@@ -7473,7 +7473,7 @@
         <v>PASS</v>
       </c>
       <c r="H266">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="267">
@@ -7499,7 +7499,7 @@
         <v>PASS</v>
       </c>
       <c r="H267">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="268">
@@ -7525,7 +7525,7 @@
         <v>PASS</v>
       </c>
       <c r="H268">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="269">
@@ -7577,7 +7577,7 @@
         <v>PASS</v>
       </c>
       <c r="H270">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="271">
@@ -7603,7 +7603,7 @@
         <v>PASS</v>
       </c>
       <c r="H271">
-        <v>33</v>
+        <v>46</v>
       </c>
     </row>
     <row r="272" xml:space="preserve">
@@ -7630,7 +7630,7 @@
         <v>PASS</v>
       </c>
       <c r="H272">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="273">
@@ -7656,7 +7656,7 @@
         <v>PASS</v>
       </c>
       <c r="H273">
-        <v>15</v>
+        <v>45</v>
       </c>
     </row>
     <row r="274">
@@ -7682,7 +7682,7 @@
         <v>PASS</v>
       </c>
       <c r="H274">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="275">
@@ -7708,7 +7708,7 @@
         <v>PASS</v>
       </c>
       <c r="H275">
-        <v>50</v>
+        <v>19</v>
       </c>
     </row>
     <row r="276">
@@ -7734,7 +7734,7 @@
         <v>PASS</v>
       </c>
       <c r="H276">
-        <v>13</v>
+        <v>35</v>
       </c>
     </row>
     <row r="277">
@@ -7760,7 +7760,7 @@
         <v>PASS</v>
       </c>
       <c r="H277">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="278">
@@ -7786,7 +7786,7 @@
         <v>PASS</v>
       </c>
       <c r="H278">
-        <v>45</v>
+        <v>16</v>
       </c>
     </row>
     <row r="279">
@@ -7812,7 +7812,7 @@
         <v>PASS</v>
       </c>
       <c r="H279">
-        <v>16</v>
+        <v>45</v>
       </c>
     </row>
     <row r="280">
@@ -7838,7 +7838,7 @@
         <v>PASS</v>
       </c>
       <c r="H280">
-        <v>20</v>
+        <v>41</v>
       </c>
     </row>
     <row r="281">
@@ -7864,7 +7864,7 @@
         <v>PASS</v>
       </c>
       <c r="H281">
-        <v>44</v>
+        <v>24</v>
       </c>
     </row>
     <row r="282">
@@ -7890,7 +7890,7 @@
         <v>PASS</v>
       </c>
       <c r="H282">
-        <v>47</v>
+        <v>29</v>
       </c>
     </row>
     <row r="283">
@@ -7916,7 +7916,7 @@
         <v>PASS</v>
       </c>
       <c r="H283">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="284">
@@ -7942,7 +7942,7 @@
         <v>PASS</v>
       </c>
       <c r="H284">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="285">
@@ -7968,7 +7968,7 @@
         <v>PASS</v>
       </c>
       <c r="H285">
-        <v>16</v>
+        <v>37</v>
       </c>
     </row>
     <row r="286">
@@ -7994,7 +7994,7 @@
         <v>PASS</v>
       </c>
       <c r="H286">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="287">
@@ -8020,7 +8020,7 @@
         <v>PASS</v>
       </c>
       <c r="H287">
-        <v>14</v>
+        <v>33</v>
       </c>
     </row>
     <row r="288">
@@ -8046,7 +8046,7 @@
         <v>PASS</v>
       </c>
       <c r="H288">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="289">
@@ -8072,7 +8072,7 @@
         <v>PASS</v>
       </c>
       <c r="H289">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="290">
@@ -8098,7 +8098,7 @@
         <v>PASS</v>
       </c>
       <c r="H290">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="291">
@@ -8124,7 +8124,7 @@
         <v>PASS</v>
       </c>
       <c r="H291">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="292">
@@ -8150,7 +8150,7 @@
         <v>PASS</v>
       </c>
       <c r="H292">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="293">
@@ -8176,7 +8176,7 @@
         <v>PASS</v>
       </c>
       <c r="H293">
-        <v>31</v>
+        <v>50</v>
       </c>
     </row>
     <row r="294">
@@ -8202,7 +8202,7 @@
         <v>PASS</v>
       </c>
       <c r="H294">
-        <v>41</v>
+        <v>29</v>
       </c>
     </row>
     <row r="295">
@@ -8228,7 +8228,7 @@
         <v>PASS</v>
       </c>
       <c r="H295">
-        <v>50</v>
+        <v>16</v>
       </c>
     </row>
     <row r="296">
@@ -8254,7 +8254,7 @@
         <v>PASS</v>
       </c>
       <c r="H296">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="297">
@@ -8280,7 +8280,7 @@
         <v>PASS</v>
       </c>
       <c r="H297">
-        <v>35</v>
+        <v>47</v>
       </c>
     </row>
     <row r="298">
@@ -8306,7 +8306,7 @@
         <v>PASS</v>
       </c>
       <c r="H298">
-        <v>34</v>
+        <v>15</v>
       </c>
     </row>
     <row r="299">
@@ -8332,7 +8332,7 @@
         <v>PASS</v>
       </c>
       <c r="H299">
-        <v>37</v>
+        <v>46</v>
       </c>
     </row>
     <row r="300" xml:space="preserve">
@@ -8359,7 +8359,7 @@
         <v>PASS</v>
       </c>
       <c r="H300">
-        <v>43</v>
+        <v>30</v>
       </c>
     </row>
     <row r="301">
@@ -8385,7 +8385,7 @@
         <v>PASS</v>
       </c>
       <c r="H301">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>